<commit_message>
Multi Page Workflow Commit Part2
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify home page loads with all approved navigation and action controls visible</t>
+          <t>Verify all approved navigation controls and action buttons are visible and enabled on the home page</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,13 +487,12 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Open the URL http://localhost/washtabui/home
-Wait for the home page to finish loading
-Observe the top navigation area and action button section</t>
+Observe the top navigation section and main action button section of the page</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Home page loads successfully with URL containing /home and the person button, back button, notification button, home navigation link, customer signup button, clean survey button, and site survey button are visible, aligned correctly, enabled, and clickable without overlapping, clipping, or broken UI elements.</t>
+          <t>['Person navigation button is visible with no broken icon or missing label', 'Back navigation button is visible with no broken icon or missing label', 'Notification button is visible with no broken icon or missing label', 'Home navigation link is visible and rendered correctly', 'Customer Signup button is visible and enabled', 'Clean Survey button is visible and enabled', 'Site Survey button is visible and enabled', 'All approved controls are clickable and displayed without overlap, truncation, or layout distortion']</t>
         </is>
       </c>
     </row>
@@ -505,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify clicking person navigation button redirects user to login page with expected URL</t>
+          <t>Verify clicking the person navigation button redirects the user to the login page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,13 +520,13 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the person navigation button once</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Person navigation button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User is redirected to the login page, the browser URL changes exactly to http://localhost/washtabui/login?data=undefined, and the login page is displayed without browser or application errors.</t>
+          <t>['Current page changes from the home page to the login page', 'Browser URL updates to http://localhost/washtabui/login?data=undefined', 'Login page content is displayed successfully', 'No application error message, blank page, or failed navigation state is displayed']</t>
         </is>
       </c>
     </row>
@@ -539,7 +538,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify customer signup button navigates to customer-search page</t>
+          <t>Verify customer signup button opens the customer-search page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,13 +554,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the customer signup button</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Customer Signup button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>User is redirected to the customer-search page and the destination page loads with visible content and no navigation, rendering, or browser errors.</t>
+          <t>['User is redirected from the home page to the customer-search page', 'Customer-search page content is fully visible after navigation', 'Target page loads without blank sections, broken UI elements, or browser errors']</t>
         </is>
       </c>
     </row>
@@ -573,7 +572,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify clean survey button navigates to vehicle-survey page</t>
+          <t>Verify clean survey button opens the vehicle-survey page</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,13 +588,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the clean survey button</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Clean Survey button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>User is redirected to the vehicle-survey page and the page content is displayed without missing sections, broken layout, or loading issues.</t>
+          <t>['User is redirected from the home page to the vehicle-survey page', 'Vehicle-survey page content becomes visible and usable', 'Navigation completes without page freeze, browser warning, or application error']</t>
         </is>
       </c>
     </row>
@@ -607,7 +606,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify site survey button navigates to survey page</t>
+          <t>Verify site survey button opens the survey page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,13 +622,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the site survey button</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Site Survey button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>User is redirected to the survey page and the survey page loads successfully with visible content and no browser or application errors.</t>
+          <t>['User is redirected from the home page to the survey page', 'Survey page content is displayed successfully', 'No unexpected popup, loading loop, or rendering issue appears during navigation']</t>
         </is>
       </c>
     </row>
@@ -641,7 +640,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify home navigation link keeps user on the home page</t>
+          <t>Verify clicking the home navigation link while already on the home page does not trigger incorrect navigation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,13 +656,13 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the home navigation link</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Home navigation link</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application remains on the home page, the browser URL continues to contain /home, and all home page controls remain visible and functional.</t>
+          <t>['User remains on the home page after clicking the Home navigation link', 'Home page URL continues to reference the home route', 'Page content reloads correctly or remains stable without duplicate overlays or navigation errors']</t>
         </is>
       </c>
     </row>
@@ -675,7 +674,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify notification button responds to user interaction without UI failure</t>
+          <t>Verify notification button interaction does not break the application UI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -691,13 +690,13 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the notification button</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Notification button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The notification button responds to the click action without page freeze, broken UI, or browser errors. Any implemented notification popup, panel, or page opens successfully.</t>
+          <t>['Notification button responds to the click action', 'Application UI remains responsive after interaction', 'If a notification panel or notification page exists, it is displayed correctly without visual corruption', 'No crash message, script error, or blank screen appears']</t>
         </is>
       </c>
     </row>
@@ -709,7 +708,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify back navigation button behavior when no previous page exists</t>
+          <t>Verify back navigation button behavior from the home page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -725,13 +724,13 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the home page directly in a fresh browser tab
-Click the back navigation button</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Back navigation button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The application handles the back action safely without displaying blank pages, crash messages, or broken navigation states. User either remains on the home page or returns to a valid browser history page if available.</t>
+          <t>['Application handles the back action without crashing', 'User is either navigated to the previous browser page or remains on the current home page', 'No blank screen, broken layout, or unresponsive state is displayed after clicking Back']</t>
         </is>
       </c>
     </row>
@@ -743,12 +742,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify all approved controls are enabled and interactable</t>
+          <t>Verify all approved controls are keyboard accessible using tab navigation</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -759,14 +758,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the home page
-Observe each approved button and link
-Interact with each control individually</t>
+          <t>Open the URL http://localhost/washtabui/home
+Press the Tab key repeatedly to move focus through the page controls
+Observe focus movement across Person, Back, Notification, Home, Customer Signup, Clean Survey, and Site Survey controls</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>All approved controls are visible, enabled, and responsive to user interaction without disabled states, delayed response, or UI failures.</t>
+          <t>['Keyboard focus reaches all approved interactive elements', 'Focused elements display a visible focus indicator or highlight', 'No approved control is skipped or inaccessible through keyboard-only navigation']</t>
         </is>
       </c>
     </row>
@@ -778,7 +777,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify browser refresh preserves visibility and functionality of home page controls</t>
+          <t>Verify direct access to the home page URL loads the correct page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -794,13 +793,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the home page
-Refresh the browser page</t>
+          <t>Launch a new browser session
+Enter the URL http://localhost/washtabui/home directly into the browser address bar
+Press Enter</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The home page reloads successfully after refresh and all approved buttons and links remain visible, enabled, and fully functional.</t>
+          <t>['Home page loads successfully in the new browser session', 'All approved navigation controls and action buttons are visible', 'No authentication warning, access denial message, or broken page content is displayed']</t>
         </is>
       </c>
     </row>
@@ -812,12 +812,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify direct access to home page URL opens the expected landing page</t>
+          <t>Verify browser refresh retains a stable home page state</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -828,13 +828,13 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Enter http://localhost/washtabui/home directly into the browser address bar
-Press Enter</t>
+          <t>Open the URL http://localhost/washtabui/home
+Refresh the browser using the refresh button or F5 key</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application opens the home page directly, the URL remains http://localhost/washtabui/home, and all approved home page controls are displayed without unexpected redirects.</t>
+          <t>['Home page reloads successfully after refresh', 'All approved controls remain visible and functional after reload', 'No duplicate controls, missing assets, stale content, or script errors appear']</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify home page layout remains usable after browser window resize</t>
+          <t>Verify browser back navigation returns the user to the home page after opening the login page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -862,14 +862,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the home page
-Resize the browser window to a smaller width
-Observe all approved controls and page layout</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Person navigation button to open the login page
+Use the browser back button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>All approved controls remain visible or accessible after resizing and the page does not display clipped buttons, overlapping text, horizontal layout corruption, or unusable navigation elements.</t>
+          <t>['Browser returns to the home page successfully', 'All home page controls are displayed correctly after returning', 'No stale loading state, navigation error, or partially rendered page is displayed']</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify browser back action returns user to home page after opening login page</t>
+          <t>Verify browser back navigation returns the user to the home page after opening the customer-search page</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -897,14 +897,14 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the person navigation button
-After the login page opens, use the browser Back action</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Customer Signup button
+Use the browser back button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The browser returns to the home page successfully and all original home page controls are visible and usable again without requiring manual refresh.</t>
+          <t>['Browser returns to the home page successfully', 'Home page buttons remain visible and functional after returning', 'No broken navigation state, duplicated content, or blank section appears']</t>
         </is>
       </c>
     </row>
@@ -916,12 +916,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify sequential navigation across multiple home page actions remains stable</t>
+          <t>Verify the home page does not display disabled or visually broken approved controls during initial load</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -932,16 +932,13 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the customer signup button and return to the home page
-Click the clean survey button and return to the home page
-Click the site survey button and return to the home page
-Click the person navigation button</t>
+          <t>Open the URL http://localhost/washtabui/home
+Observe all approved controls immediately after the page finishes loading</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Each action opens the correct destination page, returning to the home page preserves all controls and layout, and the final navigation to the login page succeeds without stale UI state, broken links, or navigation failures.</t>
+          <t>['All approved controls are fully rendered on initial page load', 'No approved control appears unintentionally disabled', 'No overlapping text, broken icons, clipped labels, or missing button text is visible']</t>
         </is>
       </c>
     </row>
@@ -953,12 +950,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify approved controls remain visible after navigating away and returning to the home page</t>
+          <t>Verify clicking non-interactive blank areas around buttons does not trigger navigation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -969,14 +966,120 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open the home page
-Navigate to the customer-search page using the customer signup button
-Return to the home page using browser navigation or application navigation</t>
+          <t>Open the URL http://localhost/washtabui/home
+Click blank areas and margins surrounding the visible action buttons without directly clicking the controls</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The home page reloads correctly after returning and all approved navigation buttons and action controls are visible, enabled, and functional without missing elements or broken layout.</t>
+          <t>['No navigation or button action is triggered when non-interactive areas are clicked', 'User remains on the home page', 'No hidden click area, unexpected redirect, or popup appears']</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT-LOGIN16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verify multiple sequential navigations from the home page work consistently without degrading the UI state</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Customer Signup button and return to the home page using browser back navigation
+Click the Clean Survey button and return to the home page
+Click the Site Survey button</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>['Each button opens the correct target page during the sequence', 'Returning to the home page preserves button visibility and functionality', 'Final navigation to the survey page succeeds without degraded performance, missing controls, or navigation failure']</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WT-LOGIN17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Verify browser forward navigation restores the previously opened page after returning to the home page</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Open the URL http://localhost/washtabui/home
+Click the Customer Signup button
+Use the browser back button to return to the home page
+Use the browser forward button</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>['Browser forward navigation returns the user to the customer-search page', 'Customer-search page content loads correctly after forward navigation', 'No stale page state, broken layout, or navigation error appears']</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WT-LOGIN18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Verify home page controls remain functional after multiple browser refresh operations</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Open the URL http://localhost/washtabui/home
+Refresh the page multiple times consecutively using the browser refresh option or F5 key
+Click the Person navigation button after the final refresh</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>['Home page reloads successfully after each refresh', 'No duplicate controls or rendering artifacts appear after repeated refreshes', 'Person navigation button remains functional and opens the login page successfully after the final refresh']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part3
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify all approved navigation controls and action buttons are visible and enabled on the home page</t>
+          <t>Verify all approved navigation and action buttons are visible on the home page</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,13 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Observe the top navigation section and main action button section of the page</t>
+          <t>Open the application home page using URL http://localhost/washtabui/home
+Observe the top and main action sections of the page
+Verify visibility of Person button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>['Person navigation button is visible with no broken icon or missing label', 'Back navigation button is visible with no broken icon or missing label', 'Notification button is visible with no broken icon or missing label', 'Home navigation link is visible and rendered correctly', 'Customer Signup button is visible and enabled', 'Clean Survey button is visible and enabled', 'Site Survey button is visible and enabled', 'All approved controls are clickable and displayed without overlap, truncation, or layout distortion']</t>
+          <t>All approved buttons are visible, fully rendered, and accessible on the home page without overlap, clipping, hidden state, or UI distortion. No browser or application error is displayed during page load.</t>
         </is>
       </c>
     </row>
@@ -504,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify clicking the person navigation button redirects the user to the login page</t>
+          <t>Verify user can navigate to login page using the Person button</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -520,13 +521,13 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Person navigation button</t>
+          <t>Open the home page
+Click the Person button once</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>['Current page changes from the home page to the login page', 'Browser URL updates to http://localhost/washtabui/login?data=undefined', 'Login page content is displayed successfully', 'No application error message, blank page, or failed navigation state is displayed']</t>
+          <t>The application redirects the user from the home page to the login page and the browser URL changes to http://localhost/washtabui/login?data=undefined. The home page controls are no longer displayed after navigation.</t>
         </is>
       </c>
     </row>
@@ -538,7 +539,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify customer signup button opens the customer-search page</t>
+          <t>Verify Customer signup button opens the customer-search page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -554,13 +555,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Customer Signup button</t>
+          <t>Open the home page
+Click the Customer signup button once</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>['User is redirected from the home page to the customer-search page', 'Customer-search page content is fully visible after navigation', 'Target page loads without blank sections, broken UI elements, or browser errors']</t>
+          <t>The application navigates away from the home page and opens the customer-search page successfully. The home page action buttons are replaced by the customer-search workflow screen without visible UI errors.</t>
         </is>
       </c>
     </row>
@@ -572,7 +573,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify clean survey button opens the vehicle-survey page</t>
+          <t>Verify Clean survey button opens the vehicle-survey page</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -588,13 +589,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Clean Survey button</t>
+          <t>Open the home page
+Click the Clean survey button once</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>['User is redirected from the home page to the vehicle-survey page', 'Vehicle-survey page content becomes visible and usable', 'Navigation completes without page freeze, browser warning, or application error']</t>
+          <t>The application navigates successfully to the vehicle-survey page and the home page interface is replaced by the vehicle-survey workflow screen without broken rendering or browser errors.</t>
         </is>
       </c>
     </row>
@@ -606,7 +607,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify site survey button opens the survey page</t>
+          <t>Verify Site survey button opens the survey page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -622,13 +623,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Site Survey button</t>
+          <t>Open the home page
+Click the Site survey button once</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>['User is redirected from the home page to the survey page', 'Survey page content is displayed successfully', 'No unexpected popup, loading loop, or rendering issue appears during navigation']</t>
+          <t>The application navigates successfully to the survey page and the user is no longer on the home page. Navigation completes without loading failures, blank pages, or UI errors.</t>
         </is>
       </c>
     </row>
@@ -640,7 +641,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify clicking the home navigation link while already on the home page does not trigger incorrect navigation</t>
+          <t>Verify Home button remains interactive on the home page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -656,13 +657,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Home navigation link</t>
+          <t>Open the home page
+Locate the Home button
+Click the Home button once</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>['User remains on the home page after clicking the Home navigation link', 'Home page URL continues to reference the home route', 'Page content reloads correctly or remains stable without duplicate overlays or navigation errors']</t>
+          <t>The Home button accepts the click interaction and the application remains stable on the home page without page corruption, browser errors, or disabled UI elements.</t>
         </is>
       </c>
     </row>
@@ -674,7 +676,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify notification button interaction does not break the application UI</t>
+          <t>Verify Notification button accepts user interaction without application failure</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -690,13 +692,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Notification button</t>
+          <t>Open the home page
+Locate the Notification button
+Click the Notification button once</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>['Notification button responds to the click action', 'Application UI remains responsive after interaction', 'If a notification panel or notification page exists, it is displayed correctly without visual corruption', 'No crash message, script error, or blank screen appears']</t>
+          <t>The Notification button responds to the click event without causing browser crashes, frozen UI, script errors, blank overlays, or unexpected navigation away from the application.</t>
         </is>
       </c>
     </row>
@@ -708,12 +711,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify back navigation button behavior from the home page</t>
+          <t>Verify Back button accepts user interaction on the home page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -724,13 +727,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Back navigation button</t>
+          <t>Open the home page
+Locate the Back button
+Click the Back button once</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>['Application handles the back action without crashing', 'User is either navigated to the previous browser page or remains on the current home page', 'No blank screen, broken layout, or unresponsive state is displayed after clicking Back']</t>
+          <t>The Back button responds to the click interaction without causing application crashes, blank screens, broken layouts, or unresponsive behavior.</t>
         </is>
       </c>
     </row>
@@ -742,12 +746,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify all approved controls are keyboard accessible using tab navigation</t>
+          <t>Verify all approved buttons are enabled and actionable on initial page load</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -758,14 +762,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Press the Tab key repeatedly to move focus through the page controls
-Observe focus movement across Person, Back, Notification, Home, Customer Signup, Clean Survey, and Site Survey controls</t>
+          <t>Open the home page
+Inspect each approved button displayed on the screen
+Verify each button appears enabled and supports pointer interaction</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>['Keyboard focus reaches all approved interactive elements', 'Focused elements display a visible focus indicator or highlight', 'No approved control is skipped or inaccessible through keyboard-only navigation']</t>
+          <t>All approved buttons appear enabled, visually interactive, and selectable. No approved button is displayed in a disabled, hidden, or inactive state on initial page load.</t>
         </is>
       </c>
     </row>
@@ -777,7 +781,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify direct access to the home page URL loads the correct page</t>
+          <t>Verify direct navigation to the home URL displays the correct home screen</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -793,14 +797,13 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Launch a new browser session
-Enter the URL http://localhost/washtabui/home directly into the browser address bar
-Press Enter</t>
+          <t>Enter http://localhost/washtabui/home directly into the browser address bar
+Press Enter to load the page</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>['Home page loads successfully in the new browser session', 'All approved navigation controls and action buttons are visible', 'No authentication warning, access denial message, or broken page content is displayed']</t>
+          <t>The browser loads the home page successfully and all approved navigation and action buttons are visible and interactive after the page finishes loading.</t>
         </is>
       </c>
     </row>
@@ -812,7 +815,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify browser refresh retains a stable home page state</t>
+          <t>Verify home page remains accessible after browser refresh</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -828,13 +831,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Refresh the browser using the refresh button or F5 key</t>
+          <t>Navigate to the home page
+Refresh the browser page
+Observe the UI after reload</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>['Home page reloads successfully after refresh', 'All approved controls remain visible and functional after reload', 'No duplicate controls, missing assets, stale content, or script errors appear']</t>
+          <t>The home page reloads successfully and all approved buttons remain visible, enabled, and interactive after the refresh. No session error, blank page, or broken UI component is displayed.</t>
         </is>
       </c>
     </row>
@@ -846,12 +850,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify browser back navigation returns the user to the home page after opening the login page</t>
+          <t>Verify no unexpected navigation occurs without user interaction on the home page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -862,224 +866,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Person navigation button to open the login page
-Use the browser back button</t>
+          <t>Open the home page
+Do not click any button for a reasonable observation period
+Observe the current page and URL</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>['Browser returns to the home page successfully', 'All home page controls are displayed correctly after returning', 'No stale loading state, navigation error, or partially rendered page is displayed']</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>WT-LOGIN13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Verify browser back navigation returns the user to the home page after opening the customer-search page</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Customer Signup button
-Use the browser back button</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>['Browser returns to the home page successfully', 'Home page buttons remain visible and functional after returning', 'No broken navigation state, duplicated content, or blank section appears']</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>WT-LOGIN14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Verify the home page does not display disabled or visually broken approved controls during initial load</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Open the URL http://localhost/washtabui/home
-Observe all approved controls immediately after the page finishes loading</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>['All approved controls are fully rendered on initial page load', 'No approved control appears unintentionally disabled', 'No overlapping text, broken icons, clipped labels, or missing button text is visible']</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>WT-LOGIN15</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Verify clicking non-interactive blank areas around buttons does not trigger navigation</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click blank areas and margins surrounding the visible action buttons without directly clicking the controls</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>['No navigation or button action is triggered when non-interactive areas are clicked', 'User remains on the home page', 'No hidden click area, unexpected redirect, or popup appears']</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>WT-LOGIN16</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Verify multiple sequential navigations from the home page work consistently without degrading the UI state</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Customer Signup button and return to the home page using browser back navigation
-Click the Clean Survey button and return to the home page
-Click the Site Survey button</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>['Each button opens the correct target page during the sequence', 'Returning to the home page preserves button visibility and functionality', 'Final navigation to the survey page succeeds without degraded performance, missing controls, or navigation failure']</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>WT-LOGIN17</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Verify browser forward navigation restores the previously opened page after returning to the home page</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Open the URL http://localhost/washtabui/home
-Click the Customer Signup button
-Use the browser back button to return to the home page
-Use the browser forward button</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>['Browser forward navigation returns the user to the customer-search page', 'Customer-search page content loads correctly after forward navigation', 'No stale page state, broken layout, or navigation error appears']</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>WT-LOGIN18</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Verify home page controls remain functional after multiple browser refresh operations</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Open the URL http://localhost/washtabui/home
-Refresh the page multiple times consecutively using the browser refresh option or F5 key
-Click the Person navigation button after the final refresh</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>['Home page reloads successfully after each refresh', 'No duplicate controls or rendering artifacts appear after repeated refreshes', 'Person navigation button remains functional and opens the login page successfully after the final refresh']</t>
+          <t>The application remains on the home page throughout the observation period. No automatic redirects, popup windows, unexpected page transitions, or URL changes occur without user interaction.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part4
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify all approved navigation and action buttons are visible on the home page</t>
+          <t>Verify all approved navigation buttons and action buttons are visible on the home page</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open the application home page using URL http://localhost/washtabui/home
-Observe the top and main action sections of the page
-Verify visibility of Person button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button</t>
+          <t>Navigate to http://localhost/washtabui/home
+Observe the home page UI without interacting with any control
+Verify the visibility of person button, back button, notification button, home button, customer signup button, clean survey button, and site survey button</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>All approved buttons are visible, fully rendered, and accessible on the home page without overlap, clipping, hidden state, or UI distortion. No browser or application error is displayed during page load.</t>
+          <t>All approved buttons and links are displayed on the home page, visually aligned without overlap or truncation, and each control is enabled and available for interaction.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify user can navigate to login page using the Person button</t>
+          <t>Verify clicking the person button navigates the user to the login page with expected URL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,13 +521,13 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the Person button once</t>
+          <t>Navigate to http://localhost/washtabui/home
+Click the person button once</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The application redirects the user from the home page to the login page and the browser URL changes to http://localhost/washtabui/login?data=undefined. The home page controls are no longer displayed after navigation.</t>
+          <t>The application redirects the user to the login page and the browser URL changes to http://localhost/washtabui/login?data=undefined with the login page loaded successfully.</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Customer signup button opens the customer-search page</t>
+          <t>Verify customer signup button opens the customer-search page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,13 +555,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the Customer signup button once</t>
+          <t>Navigate to http://localhost/washtabui/home
+Click the customer signup button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application navigates away from the home page and opens the customer-search page successfully. The home page action buttons are replaced by the customer-search workflow screen without visible UI errors.</t>
+          <t>The application redirects the user from the home page to the customer-search page and the destination page loads without UI errors or blank content.</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Clean survey button opens the vehicle-survey page</t>
+          <t>Verify clean survey button opens the vehicle-survey page</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,13 +589,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the Clean survey button once</t>
+          <t>Navigate to http://localhost/washtabui/home
+Click the clean survey button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application navigates successfully to the vehicle-survey page and the home page interface is replaced by the vehicle-survey workflow screen without broken rendering or browser errors.</t>
+          <t>The application redirects the user from the home page to the vehicle-survey page and the page content loads successfully without broken UI elements.</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Site survey button opens the survey page</t>
+          <t>Verify site survey button opens the survey page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,13 +623,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the home page
-Click the Site survey button once</t>
+          <t>Navigate to http://localhost/washtabui/home
+Click the site survey button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates successfully to the survey page and the user is no longer on the home page. Navigation completes without loading failures, blank pages, or UI errors.</t>
+          <t>The application redirects the user from the home page to the survey page and the survey page is displayed successfully.</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify Home button remains interactive on the home page</t>
+          <t>Verify home button remains functional when clicked from the home page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,14 +657,13 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the home page
-Locate the Home button
-Click the Home button once</t>
+          <t>Navigate to http://localhost/washtabui/home
+Locate and click the home button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The Home button accepts the click interaction and the application remains stable on the home page without page corruption, browser errors, or disabled UI elements.</t>
+          <t>The application remains on the home page after clicking the home button and the URL continues to display the home page address without rendering issues or unexpected redirects.</t>
         </is>
       </c>
     </row>
@@ -676,7 +675,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify Notification button accepts user interaction without application failure</t>
+          <t>Verify notification button accepts click interaction without application failure</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -692,14 +691,13 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the home page
-Locate the Notification button
-Click the Notification button once</t>
+          <t>Navigate to http://localhost/washtabui/home
+Click the notification button once</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The Notification button responds to the click event without causing browser crashes, frozen UI, script errors, blank overlays, or unexpected navigation away from the application.</t>
+          <t>The notification button responds to the click action without browser errors, application crashes, frozen UI state, or page corruption, and the application remains responsive.</t>
         </is>
       </c>
     </row>
@@ -711,7 +709,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Back button accepts user interaction on the home page</t>
+          <t>Verify back button responds to user interaction on the home page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -727,14 +725,13 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the home page
-Locate the Back button
-Click the Back button once</t>
+          <t>Navigate to http://localhost/washtabui/home
+Click the back button once</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Back button responds to the click interaction without causing application crashes, blank screens, broken layouts, or unresponsive behavior.</t>
+          <t>The back button accepts the click action without displaying browser errors, broken layouts, or unresponsive UI behavior.</t>
         </is>
       </c>
     </row>
@@ -746,12 +743,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify all approved buttons are enabled and actionable on initial page load</t>
+          <t>Verify home page remains usable after browser back navigation</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -762,14 +759,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the home page
-Inspect each approved button displayed on the screen
-Verify each button appears enabled and supports pointer interaction</t>
+          <t>Navigate to http://localhost/washtabui/home
+Click the customer signup button
+Use browser back navigation to return to the home page
+Observe the home page controls</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>All approved buttons appear enabled, visually interactive, and selectable. No approved button is displayed in a disabled, hidden, or inactive state on initial page load.</t>
+          <t>The browser returns to the home page successfully and all approved controls are visible, enabled, and responsive after navigation back to the page.</t>
         </is>
       </c>
     </row>
@@ -781,12 +779,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify direct navigation to the home URL displays the correct home screen</t>
+          <t>Verify refreshing the home page preserves approved controls and layout</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -797,13 +795,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Enter http://localhost/washtabui/home directly into the browser address bar
-Press Enter to load the page</t>
+          <t>Navigate to http://localhost/washtabui/home
+Refresh the browser page
+Observe the page after reload</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The browser loads the home page successfully and all approved navigation and action buttons are visible and interactive after the page finishes loading.</t>
+          <t>The home page reloads successfully after refresh and all approved controls remain visible, correctly aligned, and interactive without missing UI components.</t>
         </is>
       </c>
     </row>
@@ -815,12 +814,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify home page remains accessible after browser refresh</t>
+          <t>Verify user remains on the home page when no action is performed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -831,14 +830,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to the home page
-Refresh the browser page
-Observe the UI after reload</t>
+          <t>Navigate to http://localhost/washtabui/home
+Do not click any navigation or action button
+Observe the page state for several seconds</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The home page reloads successfully and all approved buttons remain visible, enabled, and interactive after the refresh. No session error, blank page, or broken UI component is displayed.</t>
+          <t>The application remains on the home page without automatic redirects, unexpected navigation, forced refresh, or disappearing UI controls.</t>
         </is>
       </c>
     </row>
@@ -850,12 +849,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify no unexpected navigation occurs without user interaction on the home page</t>
+          <t>Verify approved controls remain clickable after page refresh</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -866,14 +865,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the home page
-Do not click any button for a reasonable observation period
-Observe the current page and URL</t>
+          <t>Navigate to http://localhost/washtabui/home
+Refresh the browser page
+Click the person button after the page reload completes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application remains on the home page throughout the observation period. No automatic redirects, popup windows, unexpected page transitions, or URL changes occur without user interaction.</t>
+          <t>After refreshing the home page, the person button remains interactive and clicking it redirects the user to http://localhost/washtabui/login?data=undefined without delay or UI failure.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part8
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Home page loads successfully in guest state for an unauthenticated user</t>
+          <t>Verify Home page loads successfully in guest state for unauthenticated user</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application in a new browser session.
-Navigate to http://localhost/washtabui/home.
-Wait for the SPA Home page to finish loading.</t>
+          <t>Launch the application in a new browser session
+Navigate to http://localhost/washtabui/home
+Wait for the SPA Home page to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully without redirecting to an authenticated area. The Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are visible. No logged-in user name, authenticated identity indicator, or authenticated-only control is displayed.</t>
+          <t>The Home page loads in guest state and displays the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button in visible enabled state without displaying authenticated-only controls or logged-in user information.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify all approved guest-state controls are visible and enabled</t>
+          <t>Verify Person/Profile button opens Login page from guest Home state</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,14 +521,13 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Inspect the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button.
-Attempt to focus and interact with each control.</t>
+          <t>Open the Home page in guest state
+Click the Person/Profile button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved guest-state controls are displayed without rendering issues. Each control is enabled, accepts focus or click interaction, and does not appear hidden, blocked, disabled, or read-only.</t>
+          <t>The Login page or Login view opens from the guest Home page and the application remains in unauthenticated state until credentials are entered.</t>
         </is>
       </c>
     </row>
@@ -540,7 +539,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify clicking the Person/Profile button opens the Login page</t>
+          <t>Verify Customer signup button navigates to customer-search page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,13 +555,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Person/Profile button once.</t>
+          <t>Open the Home page in guest state
+Click the Customer signup button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Login page or Login view opens after clicking the Person/Profile button. The login experience becomes visible without duplicate overlays, page corruption, or SPA rendering issues.</t>
+          <t>The SPA navigates away from the guest Home page and displays the customer-search page content without requiring authentication.</t>
         </is>
       </c>
     </row>
@@ -574,7 +573,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Customer signup button navigates to the customer-search page</t>
+          <t>Verify Clean survey button navigates to vehicle-survey page</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -590,13 +589,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Customer signup button.</t>
+          <t>Open the Home page in guest state
+Click the Clean survey button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application navigates to the customer-search page. The destination page loads completely and remains accessible to the guest user without requiring authentication.</t>
+          <t>The SPA navigates away from the guest Home page and displays the vehicle-survey page content without requiring authentication.</t>
         </is>
       </c>
     </row>
@@ -608,7 +607,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Clean survey button navigates to the vehicle-survey page</t>
+          <t>Verify Site survey button navigates to survey page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -624,13 +623,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Clean survey button.</t>
+          <t>Open the Home page in guest state
+Click the Site survey button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates to the vehicle-survey page. The vehicle-survey view loads successfully while the session remains unauthenticated.</t>
+          <t>The SPA navigates away from the guest Home page and displays the survey page content without requiring authentication.</t>
         </is>
       </c>
     </row>
@@ -642,7 +641,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify Site survey button navigates to the survey page</t>
+          <t>Verify Back button returns user to Home page from customer-search page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -658,13 +657,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Site survey button.</t>
+          <t>Open the Home page in guest state
+Click the Customer signup button to open the customer-search page
+Click the Back button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application navigates to the survey page. The survey page loads successfully without redirecting to login or displaying an access denied state.</t>
+          <t>The application returns to the Home page guest state and the approved guest-state controls become visible and enabled again.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify Home button is visible and enabled in guest state</t>
+          <t>Verify Back button returns user to Home page from vehicle-survey page</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -692,14 +692,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Locate the Home button.
-Inspect the Home button state.</t>
+          <t>Open the Home page in guest state
+Click the Clean survey button to open the vehicle-survey page
+Click the Back button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The Home button is visible within the shared Home shell and is enabled for interaction without appearing inactive or disabled.</t>
+          <t>The application returns to the Home page guest state and the approved guest-state controls become visible and enabled again.</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Back button is visible and enabled in guest state</t>
+          <t>Verify Back button returns user to Home page from survey page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -727,14 +727,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Locate the Back button.
-Inspect the Back button state.</t>
+          <t>Open the Home page in guest state
+Click the Site survey button to open the survey page
+Click the Back button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Back button is visible within the Home page shell and is enabled for guest interaction.</t>
+          <t>The application returns to the Home page guest state and the approved guest-state controls become visible and enabled again.</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Notification button is visible and enabled in guest state</t>
+          <t>Verify Home button returns user to Home page from customer-search page</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -762,14 +762,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Locate the Notification button.
-Inspect the Notification button state.</t>
+          <t>Open the Home page in guest state
+Click the Customer signup button
+Click the Home button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Notification button is visible within the Home page shell and is enabled for guest interaction.</t>
+          <t>The application navigates back to the guest Home page and displays the approved guest-accessible controls in enabled state.</t>
         </is>
       </c>
     </row>
@@ -781,12 +781,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button remains accessible after returning from Login view</t>
+          <t>Verify Home button returns user to Home page from vehicle-survey page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -797,15 +797,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Person/Profile button to open the Login page or Login view.
-Use browser navigation or SPA navigation to return to the Home page.
-Inspect the Person/Profile button.</t>
+          <t>Open the Home page in guest state
+Click the Clean survey button
+Click the Home button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Home page returns to guest state successfully. The Person/Profile button remains visible and enabled, and no authenticated identity information appears.</t>
+          <t>The application navigates back to the guest Home page and displays the approved guest-accessible controls in enabled state.</t>
         </is>
       </c>
     </row>
@@ -817,12 +816,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify Home button interaction preserves guest-state controls</t>
+          <t>Verify Home button returns user to Home page from survey page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -833,14 +832,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Home button while already on the Home page.
-Observe the page after navigation completes.</t>
+          <t>Open the Home page in guest state
+Click the Site survey button
+Click the Home button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application remains on the Home page or reloads the Home SPA state successfully. Guest-state controls remain visible and enabled and the session remains unauthenticated.</t>
+          <t>The application navigates back to the guest Home page and displays the approved guest-accessible controls in enabled state.</t>
         </is>
       </c>
     </row>
@@ -852,12 +851,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify sequential navigation across guest-accessible feature buttons</t>
+          <t>Verify Home button behavior when already on Home page in guest state</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -868,17 +867,13 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Navigate to the customer-search page using Customer signup.
-Return to the Home page.
-Navigate to the vehicle-survey page using Clean survey.
-Return to the Home page.
-Navigate to the survey page using Site survey.</t>
+          <t>Open the Home page in guest state
+Click the Home button while already on the Home page</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Each guest-accessible feature button consistently opens its intended destination page during sequential navigation. Returning to the Home page preserves the guest state and the SPA remains stable throughout the workflow.</t>
+          <t>The application remains on the guest Home page and does not duplicate content, reload unexpectedly, or display any application error.</t>
         </is>
       </c>
     </row>
@@ -890,7 +885,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify direct navigation to the Home URL opens the guest Home state</t>
+          <t>Verify Back button behavior when user is already on initial Home page guest state</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -906,14 +901,13 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open a new browser session without an authenticated user session.
-Directly enter http://localhost/washtabui/home in the browser address bar.
-Wait for the page to load completely.</t>
+          <t>Launch the application directly to the Home page in a new guest session
+Click the Back button without performing prior page navigation</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The application opens directly to the guest Home state without redirecting to a restricted or authenticated page. Approved guest controls are visible and no authenticated identity information is displayed.</t>
+          <t>The application handles the Back button action gracefully without displaying a crash, broken SPA state, blank screen, or JavaScript error.</t>
         </is>
       </c>
     </row>
@@ -925,12 +919,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify guest-state controls remain actionable after navigating away and returning to Home</t>
+          <t>Verify Notification button is visible and enabled in guest Home state</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -941,15 +935,50 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Navigate to the customer-search page using Customer signup.
-Use available navigation to return to the Home page.
-Click the Clean survey button.</t>
+          <t>Open the Home page in guest state
+Locate the Notification button
+Click the Notification button once</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The application returns to the Home page successfully and subsequent guest navigation actions remain functional. The Clean survey button opens the vehicle-survey page correctly after returning to Home.</t>
+          <t>The Notification button is visible and enabled and the application accepts the interaction without UI breakage, navigation failure, or application instability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WT-HOME15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Verify guest-accessible feature buttons remain available after returning to Home page</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Open the Home page in guest state
+Navigate to the customer-search page using Customer signup button
+Return to Home page using the Home button
+Observe the Customer signup, Clean survey, and Site survey buttons</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>After returning to Home page, all guest-accessible feature buttons remain visible, enabled, and available for reuse without requiring page reload or authentication.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 9
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -488,12 +488,12 @@
         <is>
           <t>Launch the application in a new browser session
 Navigate to http://localhost/washtabui/home
-Wait for the SPA Home page to finish loading</t>
+Wait for the Home page to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads in guest state and displays the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button in visible enabled state without displaying authenticated-only controls or logged-in user information.</t>
+          <t>The Home page loads successfully in guest state, the browser URL contains /washtabui/home, and all approved guest-state controls are displayed without authenticated user indicators.</t>
         </is>
       </c>
     </row>
@@ -521,13 +521,13 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
+          <t>Navigate to the Home page as a guest user
 Click the Person/Profile button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Login page or Login view opens from the guest Home page and the application remains in unauthenticated state until credentials are entered.</t>
+          <t>The Login page or Login view is displayed and the guest Home state transitions into the login workflow without authenticating the user automatically.</t>
         </is>
       </c>
     </row>
@@ -555,13 +555,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
+          <t>Navigate to the Home page as a guest user
 Click the Customer signup button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The SPA navigates away from the guest Home page and displays the customer-search page content without requiring authentication.</t>
+          <t>The application navigates to the customer-search page and the customer-search workflow view is displayed successfully for a guest user.</t>
         </is>
       </c>
     </row>
@@ -589,13 +589,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
+          <t>Navigate to the Home page as a guest user
 Click the Clean survey button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The SPA navigates away from the guest Home page and displays the vehicle-survey page content without requiring authentication.</t>
+          <t>The application navigates to the vehicle-survey page and the vehicle-survey workflow is displayed while remaining in guest state.</t>
         </is>
       </c>
     </row>
@@ -623,13 +623,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
+          <t>Navigate to the Home page as a guest user
 Click the Site survey button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The SPA navigates away from the guest Home page and displays the survey page content without requiring authentication.</t>
+          <t>The application navigates to the survey page and the survey workflow is displayed successfully from the guest Home state.</t>
         </is>
       </c>
     </row>
@@ -641,12 +641,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify Back button returns user to Home page from customer-search page</t>
+          <t>Verify authenticated-only controls are not visible in guest Home state</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -657,14 +657,13 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Customer signup button to open the customer-search page
-Click the Back button</t>
+          <t>Navigate to the Home page without signing in
+Inspect the Home page shell controls and visible feature buttons</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the approved guest-state controls become visible and enabled again.</t>
+          <t>Authenticated-only controls and authenticated-only feature buttons are absent or remain inaccessible while the user is unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -676,7 +675,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify Back button returns user to Home page from vehicle-survey page</t>
+          <t>Verify Back button returns user to Home page after navigating to Customer signup page</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -692,14 +691,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Clean survey button to open the vehicle-survey page
-Click the Back button</t>
+          <t>Navigate to the Home page as a guest user
+Click the Customer signup button
+After the customer-search page opens click the Back button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the approved guest-state controls become visible and enabled again.</t>
+          <t>The application returns to the Home page guest state and all approved guest-state controls are visible again.</t>
         </is>
       </c>
     </row>
@@ -711,7 +710,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Back button returns user to Home page from survey page</t>
+          <t>Verify Home button returns user to Home page after navigating to Clean survey page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -727,14 +726,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Site survey button to open the survey page
-Click the Back button</t>
+          <t>Navigate to the Home page as a guest user
+Click the Clean survey button
+After the vehicle-survey page opens click the Home button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the approved guest-state controls become visible and enabled again.</t>
+          <t>The application returns to the Home page guest state and guest-accessible controls remain visible and enabled.</t>
         </is>
       </c>
     </row>
@@ -746,7 +745,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Home button returns user to Home page from customer-search page</t>
+          <t>Verify Home button returns user to Home page after navigating to Site survey page</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -762,14 +761,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Customer signup button
-Click the Home button</t>
+          <t>Navigate to the Home page as a guest user
+Click the Site survey button
+After the survey page opens click the Home button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The application navigates back to the guest Home page and displays the approved guest-accessible controls in enabled state.</t>
+          <t>The application returns to the Home page guest state and the Person/Profile button and guest-accessible feature buttons are displayed again.</t>
         </is>
       </c>
     </row>
@@ -781,7 +780,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Home button returns user to Home page from vehicle-survey page</t>
+          <t>Verify Back button from Login page returns to Home page guest state</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -797,14 +796,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Clean survey button
-Click the Home button</t>
+          <t>Navigate to the Home page as a guest user
+Click the Person/Profile button
+When the Login page or Login view opens click the Back button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application navigates back to the guest Home page and displays the approved guest-accessible controls in enabled state.</t>
+          <t>The Login page or Login view closes and the application returns to the Home page guest state with approved guest controls visible.</t>
         </is>
       </c>
     </row>
@@ -816,7 +815,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify Home button returns user to Home page from survey page</t>
+          <t>Verify Home button from Login page returns to Home page guest state</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -832,14 +831,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Site survey button
-Click the Home button</t>
+          <t>Navigate to the Home page as a guest user
+Click the Person/Profile button
+When the Login page or Login view opens click the Home button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application navigates back to the guest Home page and displays the approved guest-accessible controls in enabled state.</t>
+          <t>The application navigates back to the Home page guest state and no authenticated account details are displayed.</t>
         </is>
       </c>
     </row>
@@ -851,12 +850,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Home button behavior when already on Home page in guest state</t>
+          <t>Verify Notification button is visible enabled and stable in guest Home state</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -867,13 +866,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Home button while already on the Home page</t>
+          <t>Navigate to the Home page as a guest user
+Locate the Notification button
+Click the Notification button once</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application remains on the guest Home page and does not duplicate content, reload unexpectedly, or display any application error.</t>
+          <t>The Notification button remains visible and enabled and clicking it does not freeze the interface, remove guest controls, redirect unexpectedly, or display application errors.</t>
         </is>
       </c>
     </row>
@@ -885,12 +885,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Back button behavior when user is already on initial Home page guest state</t>
+          <t>Verify direct navigation to Home URL opens guest Home state</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -901,13 +901,14 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Launch the application directly to the Home page in a new guest session
-Click the Back button without performing prior page navigation</t>
+          <t>Open a fresh browser session without authentication
+Enter http://localhost/washtabui/home directly in the browser address bar
+Wait for the application to load</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The application handles the Back button action gracefully without displaying a crash, broken SPA state, blank screen, or JavaScript error.</t>
+          <t>The application opens directly into the Home page guest state and displays only guest-accessible controls and shared Home controls.</t>
         </is>
       </c>
     </row>
@@ -919,12 +920,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify Notification button is visible and enabled in guest Home state</t>
+          <t>Verify Home button behavior when already on Home page guest state</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -935,14 +936,13 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Locate the Notification button
-Click the Notification button once</t>
+          <t>Navigate to the Home page as a guest user
+Click the Home button while remaining on the Home page</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The Notification button is visible and enabled and the application accepts the interaction without UI breakage, navigation failure, or application instability.</t>
+          <t>The application remains on the Home page guest state without navigation loops, duplicate rendering, unexpected reload behavior, or disappearance of guest-state controls.</t>
         </is>
       </c>
     </row>
@@ -954,12 +954,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify guest-accessible feature buttons remain available after returning to Home page</t>
+          <t>Verify Back button behavior when guest user is already on initial Home page</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -970,15 +970,158 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Navigate to the customer-search page using Customer signup button
-Return to Home page using the Home button
+          <t>Open a fresh browser session
+Navigate directly to the Home page
+Click the Back button without prior in-application navigation</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>The application handles the Back action gracefully without crashing, exposing authenticated content, displaying script errors, or corrupting the Home page state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT-HOME16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verify guest-accessible feature buttons remain available after returning from secondary page</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Navigate to the Home page as a guest user
+Click the Customer signup button
+Use the Back button to return to the Home page
 Observe the Customer signup, Clean survey, and Site survey buttons</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>After returning to Home page, all guest-accessible feature buttons remain visible, enabled, and available for reuse without requiring page reload or authentication.</t>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>After returning to the Home page all guest-accessible feature buttons remain visible, enabled, and available for continued interaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WT-HOME17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Verify guest Home state remains unauthenticated after navigating through multiple guest workflows</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Navigate to the Home page as a guest user
+Click the Customer signup button and return to the Home page
+Click the Clean survey button and return to the Home page
+Click the Site survey button and return to the Home page</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>The user remains in guest state throughout all navigation flows and no authenticated-only control or logged-in user name becomes visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WT-HOME18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Verify Person/Profile button remains visible after returning from Login page</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Navigate to the Home page as a guest user
+Click the Person/Profile button
+Return to the Home page using the Back button
+Observe the Person/Profile button</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>The Person/Profile button is visible enabled and available for interaction after returning from the Login page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WT-HOME19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Verify guest-accessible feature buttons can be opened sequentially without application instability</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Navigate to the Home page as a guest user
+Open the Customer signup page and return to Home
+Open the Clean survey page and return to Home
+Open the Site survey page and return to Home</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Each guest-accessible workflow opens successfully and the Home page remains stable and usable after sequential navigation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 10
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Home page loads successfully in guest state for unauthenticated user</t>
+          <t>Verify Home page loads successfully in guest state from direct URL navigation</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application in a new browser session
-Navigate to http://localhost/washtabui/home
-Wait for the Home page to finish loading</t>
+          <t>Launch the application in a new browser session.
+Navigate to http://localhost/washtabui/home.
+Wait for the SPA Home page to finish loading.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state, the browser URL contains /washtabui/home, and all approved guest-state controls are displayed without authenticated user indicators.</t>
+          <t>The browser remains on the URL http://localhost/washtabui/home, the Home page loads without authentication prompts or application errors, and the guest-state controls are displayed in enabled state.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button opens Login page from guest Home state</t>
+          <t>Verify guest-state controls and guest-accessible feature buttons are visible and enabled on Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,13 +521,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Person/Profile button</t>
+          <t>Open the Home page in guest state.
+Observe the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button.
+Attempt to focus and click each control once.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Login page or Login view is displayed and the guest Home state transitions into the login workflow without authenticating the user automatically.</t>
+          <t>All approved guest-state controls and guest-accessible feature buttons are visible, enabled, keyboard focusable, and clickable without disabled styling, blocked interaction, or client-side errors.</t>
         </is>
       </c>
     </row>
@@ -539,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Customer signup button navigates to customer-search page</t>
+          <t>Verify Person/Profile button opens the Login page from guest Home state</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,13 +556,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Customer signup button</t>
+          <t>Open the Home page in guest state.
+Click the Person/Profile button.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application navigates to the customer-search page and the customer-search workflow view is displayed successfully for a guest user.</t>
+          <t>The Login page or Login view opens successfully, the Home guest-state view is replaced by the authentication entry screen, and no authenticated user controls are displayed.</t>
         </is>
       </c>
     </row>
@@ -573,7 +574,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Clean survey button navigates to vehicle-survey page</t>
+          <t>Verify Customer signup button navigates to the customer-search page</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,13 +590,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Clean survey button</t>
+          <t>Open the Home page in guest state.
+Click the Customer signup button.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application navigates to the vehicle-survey page and the vehicle-survey workflow is displayed while remaining in guest state.</t>
+          <t>The application navigates away from the Home guest-state view and displays the customer-search page without browser errors, blank content, or blocked access.</t>
         </is>
       </c>
     </row>
@@ -607,7 +608,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Site survey button navigates to survey page</t>
+          <t>Verify Clean survey button navigates to the vehicle-survey page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,13 +624,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Site survey button</t>
+          <t>Open the Home page in guest state.
+Click the Clean survey button.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates to the survey page and the survey workflow is displayed successfully from the guest Home state.</t>
+          <t>The application navigates away from the Home guest-state view and displays the vehicle-survey page without rendering failures or unauthorized access messaging.</t>
         </is>
       </c>
     </row>
@@ -641,12 +642,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify authenticated-only controls are not visible in guest Home state</t>
+          <t>Verify Site survey button navigates to the survey page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -657,13 +658,13 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to the Home page without signing in
-Inspect the Home page shell controls and visible feature buttons</t>
+          <t>Open the Home page in guest state.
+Click the Site survey button.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authenticated-only controls and authenticated-only feature buttons are absent or remain inaccessible while the user is unauthenticated.</t>
+          <t>The application navigates away from the Home guest-state view and displays the survey page successfully without application errors or blocked guest access.</t>
         </is>
       </c>
     </row>
@@ -675,7 +676,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify Back button returns user to Home page after navigating to Customer signup page</t>
+          <t>Verify Home button returns the user to Home page after navigating to Customer signup</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -691,14 +692,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Customer signup button
-After the customer-search page opens click the Back button</t>
+          <t>Open the Home page in guest state.
+Click the Customer signup button.
+After the customer-search page loads, click the Home button.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and all approved guest-state controls are visible again.</t>
+          <t>The application returns to the Home page guest state and displays the Person/Profile button, Home button, and guest-accessible feature buttons in enabled state.</t>
         </is>
       </c>
     </row>
@@ -710,7 +711,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Home button returns user to Home page after navigating to Clean survey page</t>
+          <t>Verify Back button returns the user to Home page after navigating to Clean survey</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -726,14 +727,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Clean survey button
-After the vehicle-survey page opens click the Home button</t>
+          <t>Open the Home page in guest state.
+Click the Clean survey button.
+After the vehicle-survey page loads, click the Back button.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and guest-accessible controls remain visible and enabled.</t>
+          <t>The application returns to the Home page guest state and the shared Home controls and guest-accessible feature buttons are displayed again in enabled state.</t>
         </is>
       </c>
     </row>
@@ -745,12 +746,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Home button returns user to Home page after navigating to Site survey page</t>
+          <t>Verify Home button keeps the user on the Home page when already in guest Home state</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -761,14 +762,13 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Site survey button
-After the survey page opens click the Home button</t>
+          <t>Open the Home page in guest state.
+Click the Home button while remaining on the Home page.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the Person/Profile button and guest-accessible feature buttons are displayed again.</t>
+          <t>The Home page remains loaded in guest state, no duplicate page content or overlay appears, and the page does not navigate away or reload into an invalid state.</t>
         </is>
       </c>
     </row>
@@ -780,12 +780,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Back button from Login page returns to Home page guest state</t>
+          <t>Verify Back button behavior from initial guest Home page load</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -796,14 +796,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Person/Profile button
-When the Login page or Login view opens click the Back button</t>
+          <t>Launch a fresh browser session.
+Directly navigate to http://localhost/washtabui/home.
+Click the Back button from the Home page shell.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Login page or Login view closes and the application returns to the Home page guest state with approved guest controls visible.</t>
+          <t>The application handles the Back button interaction without crashing, displaying script errors, freezing the SPA, or exposing unauthorized authenticated content.</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify Home button from Login page returns to Home page guest state</t>
+          <t>Verify Notification button is visible and interactive in guest Home state</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -831,14 +831,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Person/Profile button
-When the Login page or Login view opens click the Home button</t>
+          <t>Open the Home page in guest state.
+Locate the Notification button.
+Click the Notification button once.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application navigates back to the Home page guest state and no authenticated account details are displayed.</t>
+          <t>The Notification button is visible and enabled in guest state and accepts the click interaction without causing application crashes, visible error messages, or broken page rendering.</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Notification button is visible enabled and stable in guest Home state</t>
+          <t>Verify guest-accessible feature buttons remain enabled after returning to Home page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -866,262 +866,15 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Locate the Notification button
-Click the Notification button once</t>
+          <t>Open the Home page in guest state.
+Navigate to the customer-search page using Customer signup.
+Return to Home using the Home button.
+Observe the Customer signup, Clean survey, and Site survey buttons.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The Notification button remains visible and enabled and clicking it does not freeze the interface, remove guest controls, redirect unexpectedly, or display application errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>WT-HOME13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Verify direct navigation to Home URL opens guest Home state</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Open a fresh browser session without authentication
-Enter http://localhost/washtabui/home directly in the browser address bar
-Wait for the application to load</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>The application opens directly into the Home page guest state and displays only guest-accessible controls and shared Home controls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>WT-HOME14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Verify Home button behavior when already on Home page guest state</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Navigate to the Home page as a guest user
-Click the Home button while remaining on the Home page</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>The application remains on the Home page guest state without navigation loops, duplicate rendering, unexpected reload behavior, or disappearance of guest-state controls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>WT-HOME15</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Verify Back button behavior when guest user is already on initial Home page</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Open a fresh browser session
-Navigate directly to the Home page
-Click the Back button without prior in-application navigation</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>The application handles the Back action gracefully without crashing, exposing authenticated content, displaying script errors, or corrupting the Home page state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>WT-HOME16</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Verify guest-accessible feature buttons remain available after returning from secondary page</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Navigate to the Home page as a guest user
-Click the Customer signup button
-Use the Back button to return to the Home page
-Observe the Customer signup, Clean survey, and Site survey buttons</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>After returning to the Home page all guest-accessible feature buttons remain visible, enabled, and available for continued interaction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>WT-HOME17</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Verify guest Home state remains unauthenticated after navigating through multiple guest workflows</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Navigate to the Home page as a guest user
-Click the Customer signup button and return to the Home page
-Click the Clean survey button and return to the Home page
-Click the Site survey button and return to the Home page</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>The user remains in guest state throughout all navigation flows and no authenticated-only control or logged-in user name becomes visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>WT-HOME18</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Verify Person/Profile button remains visible after returning from Login page</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Navigate to the Home page as a guest user
-Click the Person/Profile button
-Return to the Home page using the Back button
-Observe the Person/Profile button</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>The Person/Profile button is visible enabled and available for interaction after returning from the Login page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WT-HOME19</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Verify guest-accessible feature buttons can be opened sequentially without application instability</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Navigate to the Home page as a guest user
-Open the Customer signup page and return to Home
-Open the Clean survey page and return to Home
-Open the Site survey page and return to Home</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Each guest-accessible workflow opens successfully and the Home page remains stable and usable after sequential navigation.</t>
+          <t>Customer signup, Clean survey, and Site survey buttons remain visible, enabled, and clickable after returning to the Home page from another guest-accessible page.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 17
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Home page loads successfully in guest state from the SPA landing URL</t>
+          <t>Verify Home page loads successfully in guest state for an unauthenticated user</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application in a browser.
-Navigate directly to http://localhost/washtabui/home.
-Allow the SPA Home page to finish loading.</t>
+          <t>Launch the application in a new browser session
+Navigate to http://localhost/washtabui/home
+Wait for the Home page to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state and displays the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button as visible interactive controls.</t>
+          <t>The Home page loads successfully in guest state and displays guest-accessible controls without showing authenticated user state information.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify all approved guest-state controls are visible and enabled on Home page</t>
+          <t>Verify guest-state shared Home controls are visible and enabled on initial page load</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,14 +521,13 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open http://localhost/washtabui/home as an unauthenticated user.
-Observe the Home page guest-state controls.
-Attempt to focus and interact with each approved control without navigation.</t>
+          <t>Open http://localhost/washtabui/home in a new unauthenticated browser session
+Observe the Home page controls without interacting with them</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are visible, enabled, focusable, and appear actionable in guest state.</t>
+          <t>The Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are all visible and enabled in guest state.</t>
         </is>
       </c>
     </row>
@@ -540,7 +539,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button opens the Login page from guest Home state</t>
+          <t>Verify clicking the Person/Profile button from guest Home state opens the Login page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,13 +555,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Person/Profile button once.</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Click the Person/Profile button once</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application opens the Login page or Login view from the guest-state Home page without requiring prior authentication.</t>
+          <t>The application opens the Login page or Login view from the Home page guest state.</t>
         </is>
       </c>
     </row>
@@ -574,7 +573,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Customer signup button navigates to the customer-search page</t>
+          <t>Verify clicking the Customer signup button from guest Home state opens the customer-search page</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -590,13 +589,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Customer signup button.</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Click the Customer signup button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application navigates from the guest-state Home page to the customer-search page.</t>
+          <t>The application navigates from the guest Home page to the customer-search page.</t>
         </is>
       </c>
     </row>
@@ -608,7 +607,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Clean survey button navigates to the vehicle-survey page</t>
+          <t>Verify clicking the Clean survey button from guest Home state opens the vehicle-survey page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -624,13 +623,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Clean survey button.</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Click the Clean survey button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates from the guest-state Home page to the vehicle-survey page.</t>
+          <t>The application navigates from the guest Home page to the vehicle-survey page.</t>
         </is>
       </c>
     </row>
@@ -642,7 +641,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify Site survey button navigates to the survey page</t>
+          <t>Verify clicking the Site survey button from guest Home state opens the survey page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -658,13 +657,13 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the Site survey button.</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Click the Site survey button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application navigates from the guest-state Home page to the survey page.</t>
+          <t>The application navigates from the guest Home page to the survey page.</t>
         </is>
       </c>
     </row>
@@ -676,12 +675,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify Home page remains the same SPA Home resource in guest state</t>
+          <t>Verify Person/Profile button remains enabled and responsive after returning to Home page</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -692,14 +691,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open http://localhost/washtabui/home as an unauthenticated user.
-Observe the Home page structure and shared shell controls.
-Interact with the Home button while remaining unauthenticated.</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user
+Click the Person/Profile button to open the Login page or Login view
+Use browser navigation to return to the Home page
+Click the Person/Profile button again</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application continues to display the same Home page resource in guest state without redirecting to a separate authenticated Home implementation.</t>
+          <t>The Person/Profile button remains enabled after returning to the Home page and opens the Login page or Login view again without requiring a page refresh.</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Home button is visible and enabled in guest state</t>
+          <t>Verify shared Home shell controls remain visible in guest state after navigation back to Home</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -727,14 +727,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the Home page as a guest user.
-Locate the Home button.
-Attempt to click the Home button.</t>
+          <t>Navigate to http://localhost/washtabui/home
+Click the Customer signup button to leave the Home page
+Use browser navigation or application navigation to return to the Home page
+Observe the shared Home controls</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Home button is visible and enabled, and clicking it keeps the user within the Home experience without breaking guest-state navigation.</t>
+          <t>The Back button, Notification button, Home button, and Person/Profile button are visible and enabled again after returning to the Home guest state.</t>
         </is>
       </c>
     </row>
@@ -746,7 +747,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Notification button is visible and enabled in guest state</t>
+          <t>Verify Home button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -762,14 +763,13 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Locate the Notification button.
-Attempt to interact with the Notification button.</t>
+          <t>Open the application at http://localhost/washtabui/home
+Observe the Home button state</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Notification button is visible and enabled for interaction in guest state without causing application instability.</t>
+          <t>The Home button is visible, enabled, and displayed as part of the shared Home page shell controls in guest state.</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Back button is visible and enabled in guest state</t>
+          <t>Verify Notification button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -797,14 +797,13 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Locate the Back button.
-Attempt to interact with the Back button.</t>
+          <t>Open the application at http://localhost/washtabui/home
+Observe the Notification button state</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Back button is visible and enabled in the shared Home shell while the application remains operational in guest state.</t>
+          <t>The Notification button is visible, enabled, and displayed as part of the shared Home page shell controls in guest state.</t>
         </is>
       </c>
     </row>
@@ -816,7 +815,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify guest-accessible feature buttons remain actionable before authentication</t>
+          <t>Verify Back button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -832,15 +831,119 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the Home page as a guest user.
-Click Customer signup and return to the Home page.
-Click Clean survey and return to the Home page.
-Click Site survey and return to the Home page.</t>
+          <t>Open the application at http://localhost/washtabui/home
+Observe the Back button state</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Each approved guest-accessible feature button remains enabled and successfully navigates to its supported destination while the user is unauthenticated.</t>
+          <t>The Back button is visible, enabled, and displayed as part of the shared Home page shell controls in guest state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WT-HOME12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Verify guest Home page can be refreshed without losing guest-state controls</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Refresh the browser page
+Wait for the SPA to reload</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>The Home page reloads successfully in guest state and all approved guest-accessible controls remain visible and enabled after refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WT-HOME13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Verify direct URL access to Home page always opens guest state when no authenticated session exists</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Close all browser tabs and clear the unauthenticated session
+Directly enter http://localhost/washtabui/home into the browser address bar
+Wait for the Home page to load</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>The SPA opens directly into the Home page guest state and does not redirect to an authenticated experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WT-HOME14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Verify guest-accessible feature buttons remain actionable after opening and leaving Login view</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Navigate to http://localhost/washtabui/home
+Click the Person/Profile button to open the Login page or Login view
+Return to the Home page without authenticating
+Click the Site survey button</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>The Site survey button remains enabled and successfully opens the survey page after the user returns from the Login view without signing in.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 18
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Home page loads successfully in guest state for an unauthenticated user</t>
+          <t>Verify Home page loads successfully in guest state for unauthenticated user</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state and displays guest-accessible controls without showing authenticated user state information.</t>
+          <t>The Home page loads successfully in guest state and displays the approved guest-accessible controls without showing any authenticated user identity state.</t>
         </is>
       </c>
     </row>
@@ -521,13 +521,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open http://localhost/washtabui/home in a new unauthenticated browser session
-Observe the Home page controls without interacting with them</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user
+Observe the Home page header and shell controls
+Verify the Person/Profile button, Back button, Notification button, and Home button are visible
+Verify each shared control is enabled and can receive click interaction</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are all visible and enabled in guest state.</t>
+          <t>The Person/Profile button, Back button, Notification button, and Home button are visible, enabled, and interactable in guest state.</t>
         </is>
       </c>
     </row>
@@ -539,7 +541,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify clicking the Person/Profile button from guest Home state opens the Login page</t>
+          <t>Verify guest-accessible feature buttons are visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,13 +557,16 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Click the Person/Profile button once</t>
+          <t>Navigate to the Home page as an unauthenticated user
+Locate the Customer signup button
+Locate the Clean survey button
+Locate the Site survey button
+Verify all guest-accessible feature buttons are enabled</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application opens the Login page or Login view from the Home page guest state.</t>
+          <t>Customer signup, Clean survey, and Site survey buttons are visible and enabled for guest users on the Home page.</t>
         </is>
       </c>
     </row>
@@ -573,7 +578,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify clicking the Customer signup button from guest Home state opens the customer-search page</t>
+          <t>Verify clicking the Person/Profile button opens the Login page from guest Home state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,13 +594,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Click the Customer signup button</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user
+Click the Person/Profile button
+Observe the resulting page or SPA view transition</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application navigates from the guest Home page to the customer-search page.</t>
+          <t>The application opens the Login page or Login view after the Person/Profile button is clicked from guest Home state.</t>
         </is>
       </c>
     </row>
@@ -607,7 +613,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify clicking the Clean survey button from guest Home state opens the vehicle-survey page</t>
+          <t>Verify clicking Customer signup navigates to the customer-search page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -623,13 +629,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Click the Clean survey button</t>
+          <t>Open the Home page in guest state
+Click the Customer signup button
+Observe the SPA navigation transition</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates from the guest Home page to the vehicle-survey page.</t>
+          <t>The application navigates from the guest Home page to the customer-search page after the Customer signup button is clicked.</t>
         </is>
       </c>
     </row>
@@ -641,7 +648,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify clicking the Site survey button from guest Home state opens the survey page</t>
+          <t>Verify clicking Clean survey navigates to the vehicle-survey page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -657,13 +664,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Click the Site survey button</t>
+          <t>Open the Home page in guest state
+Click the Clean survey button
+Observe the SPA navigation transition</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application navigates from the guest Home page to the survey page.</t>
+          <t>The application navigates from the guest Home page to the vehicle-survey page after the Clean survey button is clicked.</t>
         </is>
       </c>
     </row>
@@ -675,12 +683,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button remains enabled and responsive after returning to Home page</t>
+          <t>Verify clicking Site survey navigates to the survey page</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -691,15 +699,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user
-Click the Person/Profile button to open the Login page or Login view
-Use browser navigation to return to the Home page
-Click the Person/Profile button again</t>
+          <t>Open the Home page in guest state
+Click the Site survey button
+Observe the SPA navigation transition</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The Person/Profile button remains enabled after returning to the Home page and opens the Login page or Login view again without requiring a page refresh.</t>
+          <t>The application navigates from the guest Home page to the survey page after the Site survey button is clicked.</t>
         </is>
       </c>
     </row>
@@ -711,7 +718,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify shared Home shell controls remain visible in guest state after navigation back to Home</t>
+          <t>Verify Home button remains visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -727,15 +734,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home
-Click the Customer signup button to leave the Home page
-Use browser navigation or application navigation to return to the Home page
-Observe the shared Home controls</t>
+          <t>Open the Home page as a guest user
+Locate the Home button in the shared Home controls area
+Verify the Home button is enabled
+Click the Home button while already on the Home page</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Back button, Notification button, Home button, and Person/Profile button are visible and enabled again after returning to the Home guest state.</t>
+          <t>The Home button remains visible and enabled in guest state and clicking it does not break the current Home page state.</t>
         </is>
       </c>
     </row>
@@ -747,7 +754,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Home button is visible and enabled in guest state</t>
+          <t>Verify Notification button is visible and clickable in guest state</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -763,13 +770,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the application at http://localhost/washtabui/home
-Observe the Home button state</t>
+          <t>Navigate to the Home page without logging in
+Locate the Notification button
+Verify the Notification button is enabled
+Click the Notification button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Home button is visible, enabled, and displayed as part of the shared Home page shell controls in guest state.</t>
+          <t>The Notification button is visible and clickable in guest state and the application remains stable after interaction.</t>
         </is>
       </c>
     </row>
@@ -781,7 +790,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Notification button is visible and enabled in guest state</t>
+          <t>Verify Back button is visible and clickable in guest state</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -797,13 +806,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the application at http://localhost/washtabui/home
-Observe the Notification button state</t>
+          <t>Navigate to the Home page as a guest user
+Locate the Back button
+Verify the Back button is enabled
+Click the Back button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Notification button is visible, enabled, and displayed as part of the shared Home page shell controls in guest state.</t>
+          <t>The Back button is visible and enabled in guest state and clicking it does not produce an application error or broken SPA state.</t>
         </is>
       </c>
     </row>
@@ -815,12 +826,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify Back button is visible and enabled in guest state</t>
+          <t>Verify guest-accessible feature buttons remain interactable after returning to Home page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -831,13 +842,17 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the application at http://localhost/washtabui/home
-Observe the Back button state</t>
+          <t>Navigate to the Home page as a guest user
+Click the Customer signup button and verify navigation occurs
+Return to the Home page using browser navigation or Home navigation
+Click the Clean survey button
+Return to the Home page again
+Click the Site survey button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The Back button is visible, enabled, and displayed as part of the shared Home page shell controls in guest state.</t>
+          <t>Each guest-accessible feature button continues to function correctly after repeated navigation back to the Home page and each action opens its intended destination page.</t>
         </is>
       </c>
     </row>
@@ -849,7 +864,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify guest Home page can be refreshed without losing guest-state controls</t>
+          <t>Verify direct navigation to the Home URL always loads guest state for unauthenticated session</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -865,85 +880,15 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Refresh the browser page
-Wait for the SPA to reload</t>
+          <t>Open a new private or incognito browser session
+Directly enter http://localhost/washtabui/home in the browser address bar
+Wait for the SPA to finish rendering
+Inspect the visible controls on the Home page</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The Home page reloads successfully in guest state and all approved guest-accessible controls remain visible and enabled after refresh.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>WT-HOME13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Verify direct URL access to Home page always opens guest state when no authenticated session exists</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Close all browser tabs and clear the unauthenticated session
-Directly enter http://localhost/washtabui/home into the browser address bar
-Wait for the Home page to load</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>The SPA opens directly into the Home page guest state and does not redirect to an authenticated experience.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>WT-HOME14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Verify guest-accessible feature buttons remain actionable after opening and leaving Login view</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Navigate to http://localhost/washtabui/home
-Click the Person/Profile button to open the Login page or Login view
-Return to the Home page without authenticating
-Click the Site survey button</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>The Site survey button remains enabled and successfully opens the survey page after the user returns from the Login view without signing in.</t>
+          <t>Direct navigation to the Home URL in an unauthenticated session loads the guest Home state with approved guest controls visible and authenticated-only controls absent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 24
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Home page loads successfully in guest state for unauthenticated user</t>
+          <t>Verify Home page loads successfully in guest state for an unauthenticated user</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,13 +487,13 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Launch the application in a new browser session
-Navigate to http://localhost/washtabui/home
+Navigate directly to http://localhost/washtabui/home
 Wait for the Home page to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state and displays the approved guest-accessible controls without showing any authenticated user identity state.</t>
+          <t>The Home page loads successfully in guest state for an unauthenticated user and the guest-accessible Home controls are displayed without showing authenticated user indicators.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify guest-state shared Home controls are visible and enabled on initial page load</t>
+          <t>Verify all approved guest-state controls and shared Home shell controls are visible and enabled on Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,15 +521,20 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user
-Observe the Home page header and shell controls
-Verify the Person/Profile button, Back button, Notification button, and Home button are visible
-Verify each shared control is enabled and can receive click interaction</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Observe the Home page guest-state controls
+Verify the Person/Profile button is visible and enabled
+Verify the Back button is visible and enabled
+Verify the Notification button is visible and enabled
+Verify the Home button is visible and enabled
+Verify the Customer signup button is visible and enabled
+Verify the Clean survey button is visible and enabled
+Verify the Site survey button is visible and enabled</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Person/Profile button, Back button, Notification button, and Home button are visible, enabled, and interactable in guest state.</t>
+          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, clickable, and available in the Home page guest state.</t>
         </is>
       </c>
     </row>
@@ -541,7 +546,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify guest-accessible feature buttons are visible and enabled in guest state</t>
+          <t>Verify Person/Profile button navigates from Home guest state to Login page or Login view</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -557,16 +562,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as an unauthenticated user
-Locate the Customer signup button
-Locate the Clean survey button
-Locate the Site survey button
-Verify all guest-accessible feature buttons are enabled</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Person/Profile button once
+Observe the application transition</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Customer signup, Clean survey, and Site survey buttons are visible and enabled for guest users on the Home page.</t>
+          <t>The application transitions from the Home guest state to the Login page or Login view while remaining unauthenticated before login submission.</t>
         </is>
       </c>
     </row>
@@ -578,7 +581,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify clicking the Person/Profile button opens the Login page from guest Home state</t>
+          <t>Verify Customer signup button navigates to customer-search page from Home guest state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -594,14 +597,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user
-Click the Person/Profile button
-Observe the resulting page or SPA view transition</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Customer signup button
+Observe the destination page or SPA view</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application opens the Login page or Login view after the Person/Profile button is clicked from guest Home state.</t>
+          <t>The application navigates from the Home guest state to the customer-search page and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -613,7 +616,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify clicking Customer signup navigates to the customer-search page</t>
+          <t>Verify Clean survey button navigates to vehicle-survey page from Home guest state</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -629,14 +632,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Customer signup button
-Observe the SPA navigation transition</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Clean survey button
+Observe the destination page or SPA view</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates from the guest Home page to the customer-search page after the Customer signup button is clicked.</t>
+          <t>The application navigates from the Home guest state to the vehicle-survey page and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -648,7 +651,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify clicking Clean survey navigates to the vehicle-survey page</t>
+          <t>Verify Site survey button navigates to survey page from Home guest state</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -664,14 +667,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Clean survey button
-Observe the SPA navigation transition</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Site survey button
+Observe the destination page or SPA view</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application navigates from the guest Home page to the vehicle-survey page after the Clean survey button is clicked.</t>
+          <t>The application navigates from the Home guest state to the survey page and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -683,12 +686,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify clicking Site survey navigates to the survey page</t>
+          <t>Verify guest-state execution remains unauthenticated after navigating to Login view from Person/Profile button</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -699,14 +702,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Site survey button
-Observe the SPA navigation transition</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Person/Profile button
+Observe the Login page or Login view without entering credentials
+Return to the Home page guest state using browser navigation or application navigation</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application navigates from the guest Home page to the survey page after the Site survey button is clicked.</t>
+          <t>The user remains unauthenticated throughout the navigation flow and returning to Home displays the same guest-state controls without any logged-in user indicators.</t>
         </is>
       </c>
     </row>
@@ -718,7 +722,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Home button remains visible and enabled in guest state</t>
+          <t>Verify Home button remains enabled and accessible in guest state</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -734,15 +738,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the Home page as a guest user
-Locate the Home button in the shared Home controls area
-Verify the Home button is enabled
-Click the Home button while already on the Home page</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Home button while already on the Home page
+Observe the page state after the click</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Home button remains visible and enabled in guest state and clicking it does not break the current Home page state.</t>
+          <t>The Home button remains enabled and the application stays on the Home guest state without displaying an error or changing to an authenticated state.</t>
         </is>
       </c>
     </row>
@@ -754,12 +757,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Notification button is visible and clickable in guest state</t>
+          <t>Verify Back button is visible and does not expose authenticated functionality in guest state</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -770,15 +773,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to the Home page without logging in
-Locate the Notification button
-Verify the Notification button is enabled
-Click the Notification button</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Verify the Back button is visible and enabled
+Click the Back button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Notification button is visible and clickable in guest state and the application remains stable after interaction.</t>
+          <t>The Back button interaction does not expose authenticated-only functionality and the application remains within unauthenticated guest-state behavior.</t>
         </is>
       </c>
     </row>
@@ -790,12 +792,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Back button is visible and clickable in guest state</t>
+          <t>Verify repeated clicks on Customer signup button do not create duplicate customer-search transitions</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -806,15 +808,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Locate the Back button
-Verify the Back button is enabled
-Click the Back button</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Rapidly click the Customer signup button multiple times
+Observe the navigation behavior</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Back button is visible and enabled in guest state and clicking it does not produce an application error or broken SPA state.</t>
+          <t>The application transitions cleanly to the customer-search page only once without duplicate navigation layers, duplicate requests, or UI instability.</t>
         </is>
       </c>
     </row>
@@ -826,12 +827,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify guest-accessible feature buttons remain interactable after returning to Home page</t>
+          <t>Verify guest-state controls remain visible after returning to Home page from Customer signup flow</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -842,17 +843,15 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Click the Customer signup button and verify navigation occurs
-Return to the Home page using browser navigation or Home navigation
-Click the Clean survey button
-Return to the Home page again
-Click the Site survey button</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Customer signup button
+Return to the Home page guest state using browser or application navigation
+Observe the Home page controls</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Each guest-accessible feature button continues to function correctly after repeated navigation back to the Home page and each action opens its intended destination page.</t>
+          <t>The Home page returns to the guest state with the Person/Profile, Back, Notification, Home, Customer signup, Clean survey, and Site survey buttons visible and enabled.</t>
         </is>
       </c>
     </row>
@@ -864,12 +863,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify direct navigation to the Home URL always loads guest state for unauthenticated session</t>
+          <t>Verify guest-state controls remain visible after returning to Home page from Clean survey flow</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -880,15 +879,51 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open a new private or incognito browser session
-Directly enter http://localhost/washtabui/home in the browser address bar
-Wait for the SPA to finish rendering
-Inspect the visible controls on the Home page</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Clean survey button
+Return to the Home page guest state using browser or application navigation
+Observe the Home page controls</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Direct navigation to the Home URL in an unauthenticated session loads the guest Home state with approved guest controls visible and authenticated-only controls absent.</t>
+          <t>The Home page returns to the guest state with all approved guest-state buttons visible and enabled and without authenticated user indicators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WT-HOME13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Verify guest-state controls remain visible after returning to Home page from Site survey flow</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Site survey button
+Return to the Home page guest state using browser or application navigation
+Observe the Home page controls</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>The Home page returns to the guest state with all approved guest-state controls visible, enabled, and still operating in unauthenticated mode.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 28
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application in a new browser session
+          <t>Open a browser session
 Navigate directly to http://localhost/washtabui/home
-Wait for the Home page to finish loading</t>
+Wait for the Home page guest state to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state for an unauthenticated user and the guest-accessible Home controls are displayed without showing authenticated user indicators.</t>
+          <t>The Home page loads successfully in guest state while the user remains unauthenticated and the approved guest-state controls are available on the page.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify all approved guest-state controls and shared Home shell controls are visible and enabled on Home page</t>
+          <t>Verify guest-state Home controls and shared shell controls are visible and enabled</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,20 +521,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Observe the Home page guest-state controls
-Verify the Person/Profile button is visible and enabled
-Verify the Back button is visible and enabled
-Verify the Notification button is visible and enabled
-Verify the Home button is visible and enabled
-Verify the Customer signup button is visible and enabled
-Verify the Clean survey button is visible and enabled
-Verify the Site survey button is visible and enabled</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Observe the Home page after loading completes
+Verify the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are displayed
+Verify each displayed control is enabled and clickable</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, clickable, and available in the Home page guest state.</t>
+          <t>All approved guest-state controls and shared Home shell controls are visible and enabled in the guest-state Home page.</t>
         </is>
       </c>
     </row>
@@ -546,7 +541,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button navigates from Home guest state to Login page or Login view</t>
+          <t>Verify Person/Profile button navigates from Home guest state to Login page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -562,14 +557,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+          <t>Navigate to http://localhost/washtabui/home in guest state
 Click the Person/Profile button once
-Observe the application transition</t>
+Wait for the next SPA view to load</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application transitions from the Home guest state to the Login page or Login view while remaining unauthenticated before login submission.</t>
+          <t>Selecting the Person/Profile button opens the Login page or Login view while preserving unauthenticated state.</t>
         </is>
       </c>
     </row>
@@ -597,14 +592,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+          <t>Navigate to http://localhost/washtabui/home in guest state
 Click the Customer signup button
-Observe the destination page or SPA view</t>
+Wait for navigation to complete</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application navigates from the Home guest state to the customer-search page and the user remains unauthenticated.</t>
+          <t>The application transitions from the Home guest state to the customer-search page without authenticating the user.</t>
         </is>
       </c>
     </row>
@@ -632,14 +627,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+          <t>Navigate to http://localhost/washtabui/home in guest state
 Click the Clean survey button
-Observe the destination page or SPA view</t>
+Wait for the destination page to finish loading</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates from the Home guest state to the vehicle-survey page and the user remains unauthenticated.</t>
+          <t>The vehicle-survey page opens successfully from the Home guest state while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -667,14 +662,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+          <t>Navigate to http://localhost/washtabui/home in guest state
 Click the Site survey button
-Observe the destination page or SPA view</t>
+Wait for the survey page to load</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application navigates from the Home guest state to the survey page and the user remains unauthenticated.</t>
+          <t>The survey page opens successfully from the Home guest state while the session remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -686,12 +681,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify guest-state execution remains unauthenticated after navigating to Login view from Person/Profile button</t>
+          <t>Verify returning to Home guest state after navigating to Login view</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -702,15 +697,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Person/Profile button
-Observe the Login page or Login view without entering credentials
-Return to the Home page guest state using browser navigation or application navigation</t>
+          <t>Navigate to the Home page in guest state
+Click the Person/Profile button to open the Login page or Login view
+Use browser navigation or Home navigation to return to the Home page</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The user remains unauthenticated throughout the navigation flow and returning to Home displays the same guest-state controls without any logged-in user indicators.</t>
+          <t>The application returns to the Home page guest state and the approved guest-state controls remain visible and enabled.</t>
         </is>
       </c>
     </row>
@@ -722,7 +716,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Home button remains enabled and accessible in guest state</t>
+          <t>Verify returning to Home guest state after navigating to customer-search page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -738,14 +732,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Home button while already on the Home page
-Observe the page state after the click</t>
+          <t>Open the Home page in guest state
+Click the Customer signup button
+Return to the Home page using available navigation controls or browser navigation</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Home button remains enabled and the application stays on the Home guest state without displaying an error or changing to an authenticated state.</t>
+          <t>The Home page is restored in guest state and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -757,12 +751,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Back button is visible and does not expose authenticated functionality in guest state</t>
+          <t>Verify returning to Home guest state after navigating to vehicle-survey page</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -773,14 +767,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Verify the Back button is visible and enabled
-Click the Back button</t>
+          <t>Open the Home page in guest state
+Click the Clean survey button
+Return to the Home page using available navigation controls or browser navigation</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Back button interaction does not expose authenticated-only functionality and the application remains within unauthenticated guest-state behavior.</t>
+          <t>The Home page guest state is displayed again with approved guest controls still available.</t>
         </is>
       </c>
     </row>
@@ -792,12 +786,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify repeated clicks on Customer signup button do not create duplicate customer-search transitions</t>
+          <t>Verify returning to Home guest state after navigating to survey page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -808,14 +802,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Rapidly click the Customer signup button multiple times
-Observe the navigation behavior</t>
+          <t>Navigate to the Home page in guest state
+Click the Site survey button
+Return to the Home page using browser navigation or Home controls</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application transitions cleanly to the customer-search page only once without duplicate navigation layers, duplicate requests, or UI instability.</t>
+          <t>The application returns to the Home page guest state without authenticating the session.</t>
         </is>
       </c>
     </row>
@@ -827,7 +821,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify guest-state controls remain visible after returning to Home page from Customer signup flow</t>
+          <t>Verify Home button remains visible and enabled during guest-state execution</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -843,15 +837,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Customer signup button
-Return to the Home page guest state using browser or application navigation
-Observe the Home page controls</t>
+          <t>Launch the application in guest state
+Observe the Home button before and after navigating to another approved guest destination
+Return to the Home page if needed</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The Home page returns to the guest state with the Person/Profile, Back, Notification, Home, Customer signup, Clean survey, and Site survey buttons visible and enabled.</t>
+          <t>The Home button remains visible and enabled throughout guest-state navigation flows.</t>
         </is>
       </c>
     </row>
@@ -863,7 +856,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify guest-state controls remain visible after returning to Home page from Clean survey flow</t>
+          <t>Verify Back button remains visible and enabled during guest-state execution</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -879,15 +872,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Clean survey button
-Return to the Home page guest state using browser or application navigation
-Observe the Home page controls</t>
+          <t>Navigate to the Home page as a guest user
+Verify the Back button is displayed and enabled
+Navigate to an approved guest-accessible destination and use the Back button if applicable</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The Home page returns to the guest state with all approved guest-state buttons visible and enabled and without authenticated user indicators.</t>
+          <t>The Back button remains visible and actionable during guest-state navigation without exposing authenticated functionality.</t>
         </is>
       </c>
     </row>
@@ -899,7 +891,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify guest-state controls remain visible after returning to Home page from Site survey flow</t>
+          <t>Verify Notification button remains visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -915,15 +907,14 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Site survey button
-Return to the Home page guest state using browser or application navigation
-Observe the Home page controls</t>
+          <t>Launch the Home page in guest state
+Verify the Notification button is displayed
+Select the Notification button once if interaction is supported</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The Home page returns to the guest state with all approved guest-state controls visible, enabled, and still operating in unauthenticated mode.</t>
+          <t>The Notification button is visible and enabled in guest state and does not transition the session into an authenticated state.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 29
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open a browser session
-Navigate directly to http://localhost/washtabui/home
+          <t>Launch the application in a new browser session
+Navigate to http://localhost/washtabui/home
 Wait for the Home page guest state to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state while the user remains unauthenticated and the approved guest-state controls are available on the page.</t>
+          <t>The Home page loads successfully in guest state while the user remains unauthenticated and the approved guest-state controls are available on the shared Home page.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify guest-state Home controls and shared shell controls are visible and enabled</t>
+          <t>Verify all approved guest-state buttons and shared Home shell controls are visible and enabled on Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,15 +521,20 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Home page after loading completes
-Verify the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are displayed
-Verify each displayed control is enabled and clickable</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Observe the Home page in guest state
+Verify the Person/Profile button is visible and enabled
+Verify the Back button is visible and enabled
+Verify the Notification button is visible and enabled
+Verify the Home button is visible and enabled
+Verify the Customer signup button is visible and enabled
+Verify the Clean survey button is visible and enabled
+Verify the Site survey button is visible and enabled</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved guest-state controls and shared Home shell controls are visible and enabled in the guest-state Home page.</t>
+          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, and actionable on the Home page guest state.</t>
         </is>
       </c>
     </row>
@@ -541,7 +546,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button navigates from Home guest state to Login page</t>
+          <t>Verify Person/Profile button navigates from Home guest state to Login page or Login view</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -557,14 +562,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state
-Click the Person/Profile button once
-Wait for the next SPA view to load</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Verify the Home page is displayed in guest state
+Select the Person/Profile button once</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Selecting the Person/Profile button opens the Login page or Login view while preserving unauthenticated state.</t>
+          <t>The application transitions from the Home guest state to the Login page or Login view while maintaining unauthenticated state.</t>
         </is>
       </c>
     </row>
@@ -576,7 +581,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Customer signup button navigates to customer-search page from Home guest state</t>
+          <t>Verify Customer signup button navigates from Home guest state to customer-search page</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -592,14 +597,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state
-Click the Customer signup button
-Wait for navigation to complete</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Verify the Home page guest state is visible
+Select the Customer signup button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application transitions from the Home guest state to the customer-search page without authenticating the user.</t>
+          <t>The customer-search page opens from the Home guest state and the session remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -611,7 +616,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Clean survey button navigates to vehicle-survey page from Home guest state</t>
+          <t>Verify Clean survey button navigates from Home guest state to vehicle-survey page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -627,14 +632,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state
-Click the Clean survey button
-Wait for the destination page to finish loading</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Verify the Home page guest state is visible
+Select the Clean survey button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The vehicle-survey page opens successfully from the Home guest state while the user remains unauthenticated.</t>
+          <t>The vehicle-survey page opens from the Home guest state and the session remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -646,7 +651,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify Site survey button navigates to survey page from Home guest state</t>
+          <t>Verify Site survey button navigates from Home guest state to survey page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -662,14 +667,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state
-Click the Site survey button
-Wait for the survey page to load</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Verify the Home page guest state is visible
+Select the Site survey button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The survey page opens successfully from the Home guest state while the session remains unauthenticated.</t>
+          <t>The survey page opens from the Home guest state and the session remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -681,7 +686,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify returning to Home guest state after navigating to Login view</t>
+          <t>Verify navigation back to Home guest state after opening Login view from Person/Profile button</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -697,14 +702,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to the Home page in guest state
-Click the Person/Profile button to open the Login page or Login view
-Use browser navigation or Home navigation to return to the Home page</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Select the Person/Profile button to open the Login page or Login view
+Use browser back navigation or approved application navigation to return to the Home page</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the approved guest-state controls remain visible and enabled.</t>
+          <t>The application returns to the Home page guest state and the approved guest-state controls remain visible and enabled without authenticating the user.</t>
         </is>
       </c>
     </row>
@@ -716,7 +721,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify returning to Home guest state after navigating to customer-search page</t>
+          <t>Verify navigation back to Home guest state after opening customer-search page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -732,14 +737,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Customer signup button
-Return to the Home page using available navigation controls or browser navigation</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Select the Customer signup button
+Use browser back navigation or approved application navigation to return to the Home page</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Home page is restored in guest state and the user remains unauthenticated.</t>
+          <t>The application returns to the Home page guest state and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -751,7 +756,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify returning to Home guest state after navigating to vehicle-survey page</t>
+          <t>Verify navigation back to Home guest state after opening vehicle-survey page</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -767,14 +772,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Clean survey button
-Return to the Home page using available navigation controls or browser navigation</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Select the Clean survey button
+Use browser back navigation or approved application navigation to return to the Home page</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Home page guest state is displayed again with approved guest controls still available.</t>
+          <t>The application returns to the Home page guest state and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -786,7 +791,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify returning to Home guest state after navigating to survey page</t>
+          <t>Verify navigation back to Home guest state after opening survey page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -802,14 +807,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to the Home page in guest state
-Click the Site survey button
-Return to the Home page using browser navigation or Home controls</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Select the Site survey button
+Use browser back navigation or approved application navigation to return to the Home page</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state without authenticating the session.</t>
+          <t>The application returns to the Home page guest state and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -821,12 +826,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify Home button remains visible and enabled during guest-state execution</t>
+          <t>Verify repeated clicking of Person/Profile button does not create broken navigation state</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -837,14 +842,13 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Launch the application in guest state
-Observe the Home button before and after navigating to another approved guest destination
-Return to the Home page if needed</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Rapidly click the Person/Profile button multiple times before navigation completes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The Home button remains visible and enabled throughout guest-state navigation flows.</t>
+          <t>Only the Login page or Login view is opened and the application does not display duplicate overlays, broken rendering, or inconsistent navigation behavior.</t>
         </is>
       </c>
     </row>
@@ -856,7 +860,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Back button remains visible and enabled during guest-state execution</t>
+          <t>Verify Home button remains visible and enabled throughout guest-state workflow navigation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -872,14 +876,16 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to the Home page as a guest user
-Verify the Back button is displayed and enabled
-Navigate to an approved guest-accessible destination and use the Back button if applicable</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Verify the Home button is visible and enabled in guest state
+Navigate to the Login page or Login view using the Person/Profile button
+Return to the Home page guest state
+Verify the Home button remains visible and enabled</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The Back button remains visible and actionable during guest-state navigation without exposing authenticated functionality.</t>
+          <t>The Home button remains consistently visible and enabled during guest-state navigation flows.</t>
         </is>
       </c>
     </row>
@@ -891,7 +897,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Notification button remains visible and enabled in guest state</t>
+          <t>Verify Notification button remains visible and enabled throughout guest-state workflow</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -907,14 +913,51 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Launch the Home page in guest state
-Verify the Notification button is displayed
-Select the Notification button once if interaction is supported</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Verify the Notification button is visible and enabled
+Navigate to one guest-accessible destination and return to the Home page
+Verify the Notification button remains visible and enabled</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The Notification button is visible and enabled in guest state and does not transition the session into an authenticated state.</t>
+          <t>The Notification button remains visible and enabled throughout guest-state navigation without exposing authenticated-only functionality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WT-HOME14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Verify Back button remains visible and enabled throughout guest-state workflow</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Launch the application and navigate to http://localhost/washtabui/home
+Verify the Back button is visible and enabled
+Navigate to one guest-accessible destination and return to the Home page
+Verify the Back button remains visible and enabled</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>The Back button remains visible and enabled throughout guest-state navigation without changing the user authentication state.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 30
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -486,14 +486,15 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application in a new browser session
+          <t>Open a browser session
 Navigate to http://localhost/washtabui/home
-Wait for the Home page guest state to finish loading</t>
+Wait for the Home page to finish loading
+Observe the displayed Home page state without performing login</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state while the user remains unauthenticated and the approved guest-state controls are available on the shared Home page.</t>
+          <t>The application loads the shared Home page in guest state, the Home shell is visible, and the session remains unauthenticated without any logged-in user indicators displayed.</t>
         </is>
       </c>
     </row>
@@ -505,7 +506,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify all approved guest-state buttons and shared Home shell controls are visible and enabled on Home page</t>
+          <t>Verify guest-state controls and shared Home shell controls are visible and enabled on Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,20 +522,20 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Observe the Home page in guest state
-Verify the Person/Profile button is visible and enabled
-Verify the Back button is visible and enabled
-Verify the Notification button is visible and enabled
-Verify the Home button is visible and enabled
-Verify the Customer signup button is visible and enabled
-Verify the Clean survey button is visible and enabled
-Verify the Site survey button is visible and enabled</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Verify the Person/Profile button is visible
+Verify the Back button is visible
+Verify the Notification button is visible
+Verify the Home button is visible
+Verify the Customer signup button is visible
+Verify the Clean survey button is visible
+Verify the Site survey button is visible
+Verify each displayed button is enabled and clickable</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, and actionable on the Home page guest state.</t>
+          <t>The Person/Profile, Back, Notification, Home, Customer signup, Clean survey, and Site survey buttons are all visible, enabled, and ready for interaction while the Home page remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -562,14 +563,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Home page is displayed in guest state
-Select the Person/Profile button once</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Person/Profile button once
+Observe the resulting navigation state</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application transitions from the Home guest state to the Login page or Login view while maintaining unauthenticated state.</t>
+          <t>Selecting the Person/Profile button transitions the application from Home guest state to the Login page or Login view while preserving unauthenticated status.</t>
         </is>
       </c>
     </row>
@@ -581,7 +582,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Customer signup button navigates from Home guest state to customer-search page</t>
+          <t>Verify Customer signup button navigates to customer-search page from Home guest state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -597,14 +598,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Home page guest state is visible
-Select the Customer signup button</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Customer signup button
+Observe the destination page or view</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The customer-search page opens from the Home guest state and the session remains unauthenticated.</t>
+          <t>Clicking the Customer signup button opens the customer-search page and the application remains in an unauthenticated state.</t>
         </is>
       </c>
     </row>
@@ -616,7 +617,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Clean survey button navigates from Home guest state to vehicle-survey page</t>
+          <t>Verify Clean survey button navigates to vehicle-survey page from Home guest state</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -632,14 +633,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Home page guest state is visible
-Select the Clean survey button</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Clean survey button
+Observe the destination page or view</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The vehicle-survey page opens from the Home guest state and the session remains unauthenticated.</t>
+          <t>Clicking the Clean survey button opens the vehicle-survey page and the application remains in guest-accessible unauthenticated mode.</t>
         </is>
       </c>
     </row>
@@ -651,7 +652,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify Site survey button navigates from Home guest state to survey page</t>
+          <t>Verify Site survey button navigates to survey page from Home guest state</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -667,14 +668,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Home page guest state is visible
-Select the Site survey button</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Site survey button
+Observe the destination page or view</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The survey page opens from the Home guest state and the session remains unauthenticated.</t>
+          <t>Clicking the Site survey button opens the survey page while the user session remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -702,14 +703,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Select the Person/Profile button to open the Login page or Login view
-Use browser back navigation or approved application navigation to return to the Home page</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Person/Profile button to open the Login page or Login view
+Use browser navigation or available application navigation to return to the Home page
+Observe the Home page state after returning</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the approved guest-state controls remain visible and enabled without authenticating the user.</t>
+          <t>The application returns to the shared Home page in guest state and all approved guest-state controls remain visible and enabled without authenticating the user.</t>
         </is>
       </c>
     </row>
@@ -737,14 +739,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Select the Customer signup button
-Use browser back navigation or approved application navigation to return to the Home page</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Customer signup button
+Return to the Home page using browser navigation or application navigation
+Observe the returned Home page state</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the user remains unauthenticated.</t>
+          <t>The application returns to the Home page in guest state with approved guest-accessible buttons still visible and enabled.</t>
         </is>
       </c>
     </row>
@@ -772,14 +775,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Select the Clean survey button
-Use browser back navigation or approved application navigation to return to the Home page</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Clean survey button
+Return to the Home page
+Observe the returned Home guest state</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the user remains unauthenticated.</t>
+          <t>The Home page reloads or becomes visible again in guest state and no authenticated user controls become available.</t>
         </is>
       </c>
     </row>
@@ -807,14 +811,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Select the Site survey button
-Use browser back navigation or approved application navigation to return to the Home page</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Site survey button
+Return to the Home page
+Observe the returned Home page state</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the user remains unauthenticated.</t>
+          <t>The application returns to the Home page guest state and the user remains unauthenticated throughout the workflow.</t>
         </is>
       </c>
     </row>
@@ -826,7 +831,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify repeated clicking of Person/Profile button does not create broken navigation state</t>
+          <t>Verify repeated clicking of Person/Profile button does not create inconsistent navigation state</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -842,13 +847,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Rapidly click the Person/Profile button multiple times before navigation completes</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Rapidly click the Person/Profile button multiple times
+Observe the resulting application state</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Only the Login page or Login view is opened and the application does not display duplicate overlays, broken rendering, or inconsistent navigation behavior.</t>
+          <t>The application opens only the Login page or Login view without duplicated overlays, broken navigation, or unintended authenticated state changes.</t>
         </is>
       </c>
     </row>
@@ -860,7 +866,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Home button remains visible and enabled throughout guest-state workflow navigation</t>
+          <t>Verify Home button remains visible and enabled during guest-state execution</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -876,16 +882,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Home button is visible and enabled in guest state
-Navigate to the Login page or Login view using the Person/Profile button
-Return to the Home page guest state
-Verify the Home button remains visible and enabled</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Observe the Home button on the shared Home shell
+Click the Home button while already on the Home page</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The Home button remains consistently visible and enabled during guest-state navigation flows.</t>
+          <t>The Home button is visible and enabled, and clicking it while on the Home page does not break the guest-state session or navigate to an unexpected page.</t>
         </is>
       </c>
     </row>
@@ -897,7 +901,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Notification button remains visible and enabled throughout guest-state workflow</t>
+          <t>Verify Notification button remains visible and enabled during guest-state execution</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -913,15 +917,15 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Notification button is visible and enabled
-Navigate to one guest-accessible destination and return to the Home page
-Verify the Notification button remains visible and enabled</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Observe the Notification button
+Click the Notification button once
+Observe the resulting UI behavior</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The Notification button remains visible and enabled throughout guest-state navigation without exposing authenticated-only functionality.</t>
+          <t>The Notification button is visible and enabled and interacting with it does not expose authenticated-only functionality or change the user to an authenticated state.</t>
         </is>
       </c>
     </row>
@@ -933,7 +937,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify Back button remains visible and enabled throughout guest-state workflow</t>
+          <t>Verify Back button remains visible and enabled during guest-state execution</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -949,15 +953,15 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Back button is visible and enabled
-Navigate to one guest-accessible destination and return to the Home page
-Verify the Back button remains visible and enabled</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Observe the Back button
+Click the Back button once
+Observe the resulting application behavior</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The Back button remains visible and enabled throughout guest-state navigation without changing the user authentication state.</t>
+          <t>The Back button is visible and enabled and interacting with it does not expose authenticated-only content or corrupt the guest-state navigation flow.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 31
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -488,13 +488,12 @@
         <is>
           <t>Open a browser session
 Navigate to http://localhost/washtabui/home
-Wait for the Home page to finish loading
-Observe the displayed Home page state without performing login</t>
+Wait for the Home page to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application loads the shared Home page in guest state, the Home shell is visible, and the session remains unauthenticated without any logged-in user indicators displayed.</t>
+          <t>The shared Home page loads successfully in guest state while the user remains unauthenticated and guest-accessible controls are displayed without any logged-in user identity visible.</t>
         </is>
       </c>
     </row>
@@ -506,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify guest-state controls and shared Home shell controls are visible and enabled on Home page</t>
+          <t>Verify Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -523,19 +522,19 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Verify the Person/Profile button is visible
-Verify the Back button is visible
-Verify the Notification button is visible
-Verify the Home button is visible
-Verify the Customer signup button is visible
-Verify the Clean survey button is visible
-Verify the Site survey button is visible
-Verify each displayed button is enabled and clickable</t>
+Observe the Home page guest-state controls
+Verify the Person/Profile button is visible and enabled
+Verify the Back button is visible and enabled
+Verify the Notification button is visible and enabled
+Verify the Home button is visible and enabled
+Verify the Customer signup button is visible and enabled
+Verify the Clean survey button is visible and enabled
+Verify the Site survey button is visible and enabled</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Person/Profile, Back, Notification, Home, Customer signup, Clean survey, and Site survey buttons are all visible, enabled, and ready for interaction while the Home page remains in guest state.</t>
+          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, and actionable while the application remains in Home guest state.</t>
         </is>
       </c>
     </row>
@@ -547,7 +546,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button navigates from Home guest state to Login page or Login view</t>
+          <t>Verify clicking the Person/Profile button from Home guest state opens the Login page or Login view</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -570,7 +569,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Selecting the Person/Profile button transitions the application from Home guest state to the Login page or Login view while preserving unauthenticated status.</t>
+          <t>The application transitions from the Home guest state to the Login page or Login view while the navigation originates from the Home page resource.</t>
         </is>
       </c>
     </row>
@@ -582,7 +581,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Customer signup button navigates to customer-search page from Home guest state</t>
+          <t>Verify returning to Home guest state after opening the Login view keeps guest controls available</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -599,13 +598,14 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Customer signup button
-Observe the destination page or view</t>
+Click the Person/Profile button to open the Login page or Login view
+Use browser back navigation or approved application navigation to return to Home
+Observe the Home page state after returning</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Clicking the Customer signup button opens the customer-search page and the application remains in an unauthenticated state.</t>
+          <t>The application returns to the shared Home page in guest state and the approved guest-state controls remain visible and enabled without authenticating the user.</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Clean survey button navigates to vehicle-survey page from Home guest state</t>
+          <t>Verify clicking the Customer signup button from Home guest state opens the customer-search page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -634,13 +634,13 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Clean survey button
-Observe the destination page or view</t>
+Click the Customer signup button
+Observe the destination page</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Clicking the Clean survey button opens the vehicle-survey page and the application remains in guest-accessible unauthenticated mode.</t>
+          <t>The application transitions from the Home guest state to the customer-search page while remaining unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify Site survey button navigates to survey page from Home guest state</t>
+          <t>Verify clicking the Clean survey button from Home guest state opens the vehicle-survey page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,13 +669,13 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Site survey button
-Observe the destination page or view</t>
+Click the Clean survey button
+Observe the destination page</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Clicking the Site survey button opens the survey page while the user session remains unauthenticated.</t>
+          <t>The application transitions from the Home guest state to the vehicle-survey page while remaining unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening Login view from Person/Profile button</t>
+          <t>Verify clicking the Site survey button from Home guest state opens the survey page</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -704,14 +704,13 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Person/Profile button to open the Login page or Login view
-Use browser navigation or available application navigation to return to the Home page
-Observe the Home page state after returning</t>
+Click the Site survey button
+Observe the destination page</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application returns to the shared Home page in guest state and all approved guest-state controls remain visible and enabled without authenticating the user.</t>
+          <t>The application transitions from the Home guest state to the survey page while remaining unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -723,7 +722,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening customer-search page</t>
+          <t>Verify Home button remains visible and enabled while already on the Home guest state</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -740,14 +739,13 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Customer signup button
-Return to the Home page using browser navigation or application navigation
-Observe the returned Home page state</t>
+Verify the Home button is visible and enabled
+Click the Home button while already on the Home page</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in guest state with approved guest-accessible buttons still visible and enabled.</t>
+          <t>The Home button remains actionable and the application stays on the shared Home page in guest state without errors or unexpected redirects.</t>
         </is>
       </c>
     </row>
@@ -759,7 +757,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening vehicle-survey page</t>
+          <t>Verify Back button is visible and enabled in Home guest state before any additional navigation</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -776,14 +774,12 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Clean survey button
-Return to the Home page
-Observe the returned Home guest state</t>
+Observe the Back button state without performing any prior navigation</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Home page reloads or becomes visible again in guest state and no authenticated user controls become available.</t>
+          <t>The Back button is visible and enabled as part of the shared Home shell controls in guest state.</t>
         </is>
       </c>
     </row>
@@ -795,7 +791,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening survey page</t>
+          <t>Verify Notification button is visible and enabled in Home guest state for unauthenticated users</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -812,156 +808,13 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Site survey button
-Return to the Home page
-Observe the returned Home page state</t>
+Observe the Notification button
+Attempt a single click on the Notification button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the user remains unauthenticated throughout the workflow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>WT-HOME11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Verify repeated clicking of Person/Profile button does not create inconsistent navigation state</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Rapidly click the Person/Profile button multiple times
-Observe the resulting application state</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>The application opens only the Login page or Login view without duplicated overlays, broken navigation, or unintended authenticated state changes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>WT-HOME12</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Verify Home button remains visible and enabled during guest-state execution</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Home button on the shared Home shell
-Click the Home button while already on the Home page</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>The Home button is visible and enabled, and clicking it while on the Home page does not break the guest-state session or navigate to an unexpected page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>WT-HOME13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Verify Notification button remains visible and enabled during guest-state execution</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Notification button
-Click the Notification button once
-Observe the resulting UI behavior</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>The Notification button is visible and enabled and interacting with it does not expose authenticated-only functionality or change the user to an authenticated state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>WT-HOME14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Verify Back button remains visible and enabled during guest-state execution</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Back button
-Click the Back button once
-Observe the resulting application behavior</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>The Back button is visible and enabled and interacting with it does not expose authenticated-only content or corrupt the guest-state navigation flow.</t>
+          <t>The Notification button is visible and enabled in guest state and interacting with it does not authenticate the user or expose authenticated-only controls.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 32
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -488,12 +488,12 @@
         <is>
           <t>Open a browser session
 Navigate to http://localhost/washtabui/home
-Wait for the Home page to finish loading</t>
+Wait for the Home page guest-state view to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The shared Home page loads successfully in guest state while the user remains unauthenticated and guest-accessible controls are displayed without any logged-in user identity visible.</t>
+          <t>The shared Home page loads successfully in guest state while the user remains unauthenticated, and guest-accessible controls are displayed without any authenticated user indicators.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are visible and enabled in guest state</t>
+          <t>Verify guest-state Home controls are visible and enabled on initial page load</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,20 +521,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Home page guest-state controls
-Verify the Person/Profile button is visible and enabled
-Verify the Back button is visible and enabled
-Verify the Notification button is visible and enabled
-Verify the Home button is visible and enabled
-Verify the Customer signup button is visible and enabled
-Verify the Clean survey button is visible and enabled
-Verify the Site survey button is visible and enabled</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Observe the Home page controls after the page finishes loading
+Verify the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are displayed
+Attempt to focus and click each displayed control once</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, and actionable while the application remains in Home guest state.</t>
+          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, focusable, and actionable from the Home page guest state.</t>
         </is>
       </c>
     </row>
@@ -546,7 +541,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify clicking the Person/Profile button from Home guest state opens the Login page or Login view</t>
+          <t>Verify navigation from Person/Profile button opens the Login page or Login view</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -562,14 +557,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Person/Profile button once
-Observe the resulting navigation state</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Person/Profile button from the Home page guest state
+Observe the destination view after navigation completes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application transitions from the Home guest state to the Login page or Login view while the navigation originates from the Home page resource.</t>
+          <t>Selecting the Person/Profile button transitions the application from the Home guest state to the Login page or Login view while preserving unauthenticated status.</t>
         </is>
       </c>
     </row>
@@ -581,7 +576,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify returning to Home guest state after opening the Login view keeps guest controls available</t>
+          <t>Verify navigation from Customer signup button opens the customer-search page</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -597,15 +592,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Person/Profile button to open the Login page or Login view
-Use browser back navigation or approved application navigation to return to Home
-Observe the Home page state after returning</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Customer signup button
+Observe the destination page after navigation completes</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application returns to the shared Home page in guest state and the approved guest-state controls remain visible and enabled without authenticating the user.</t>
+          <t>Selecting the Customer signup button transitions the application from the Home guest state to the customer-search page without authenticating the user.</t>
         </is>
       </c>
     </row>
@@ -617,7 +611,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify clicking the Customer signup button from Home guest state opens the customer-search page</t>
+          <t>Verify navigation from Clean survey button opens the vehicle-survey page</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -633,14 +627,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Customer signup button
-Observe the destination page</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Clean survey button
+Observe the destination page after navigation completes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application transitions from the Home guest state to the customer-search page while remaining unauthenticated.</t>
+          <t>Selecting the Clean survey button transitions the application from the Home guest state to the vehicle-survey page without changing the unauthenticated session state.</t>
         </is>
       </c>
     </row>
@@ -652,7 +646,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify clicking the Clean survey button from Home guest state opens the vehicle-survey page</t>
+          <t>Verify navigation from Site survey button opens the survey page</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -668,14 +662,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Clean survey button
-Observe the destination page</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Site survey button
+Observe the destination page after navigation completes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application transitions from the Home guest state to the vehicle-survey page while remaining unauthenticated.</t>
+          <t>Selecting the Site survey button transitions the application from the Home guest state to the survey page while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -687,7 +681,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify clicking the Site survey button from Home guest state opens the survey page</t>
+          <t>Verify returning to the Home page preserves guest-state behavior after opening the Login view</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -703,14 +697,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Site survey button
-Observe the destination page</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Person/Profile button to open the Login page or Login view
+Use browser back navigation or the application Home navigation to return to the Home page
+Observe the Home page after returning</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application transitions from the Home guest state to the survey page while remaining unauthenticated.</t>
+          <t>The application returns to the shared Home page in guest state, approved guest controls remain visible and enabled, and the user is still unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -722,7 +717,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Home button remains visible and enabled while already on the Home guest state</t>
+          <t>Verify Home button remains visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -738,14 +733,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Verify the Home button is visible and enabled
-Click the Home button while already on the Home page</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Locate the Home button in the shared Home shell
+Select the Home button while already on the Home page</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Home button remains actionable and the application stays on the shared Home page in guest state without errors or unexpected redirects.</t>
+          <t>The Home button is visible and enabled in guest state and selecting it keeps the application on the Home page guest state without authentication changes.</t>
         </is>
       </c>
     </row>
@@ -757,7 +752,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Back button is visible and enabled in Home guest state before any additional navigation</t>
+          <t>Verify Notification button remains visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -773,13 +768,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Back button state without performing any prior navigation</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Locate the Notification button in the shared Home shell
+Click the Notification button once</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Back button is visible and enabled as part of the shared Home shell controls in guest state.</t>
+          <t>The Notification button is visible and enabled in guest state, and clicking it does not expose authenticated-only capabilities or change the unauthenticated session state.</t>
         </is>
       </c>
     </row>
@@ -791,7 +787,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Notification button is visible and enabled in Home guest state for unauthenticated users</t>
+          <t>Verify Back button remains visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -807,14 +803,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Notification button
-Attempt a single click on the Notification button</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Locate the Back button in the shared Home shell
+Click the Back button from the Home page guest state</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Notification button is visible and enabled in guest state and interacting with it does not authenticate the user or expose authenticated-only controls.</t>
+          <t>The Back button is visible and enabled in guest state and does not expose authenticated-only content or cause unauthorized navigation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 33
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -488,12 +488,12 @@
         <is>
           <t>Open a browser session
 Navigate to http://localhost/washtabui/home
-Wait for the Home page guest-state view to finish loading</t>
+Wait for the Home page guest state to finish loading</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The shared Home page loads successfully in guest state while the user remains unauthenticated, and guest-accessible controls are displayed without any authenticated user indicators.</t>
+          <t>The Home page loads successfully in guest state while the user remains unauthenticated and the shared Home page shell is visible.</t>
         </is>
       </c>
     </row>
@@ -521,15 +521,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Observe the Home page controls after the page finishes loading
-Verify the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are displayed
-Attempt to focus and click each displayed control once</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Observe the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button
+Attempt to focus and click each visible control once</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, focusable, and actionable from the Home page guest state.</t>
+          <t>The Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are visible, enabled, focusable, and actionable in guest state.</t>
         </is>
       </c>
     </row>
@@ -541,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify navigation from Person/Profile button opens the Login page or Login view</t>
+          <t>Verify navigation from Person/Profile button opens the Login page or Login view from Home guest state</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -557,14 +556,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Person/Profile button from the Home page guest state
-Observe the destination view after navigation completes</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Person/Profile button once
+Observe the application transition</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Selecting the Person/Profile button transitions the application from the Home guest state to the Login page or Login view while preserving unauthenticated status.</t>
+          <t>Selecting the Person/Profile button transitions the application from Home guest state to the Login page or Login view while preserving unauthenticated state.</t>
         </is>
       </c>
     </row>
@@ -592,14 +591,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Customer signup button
-Observe the destination page after navigation completes</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Customer signup button once
+Observe the destination view</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Selecting the Customer signup button transitions the application from the Home guest state to the customer-search page without authenticating the user.</t>
+          <t>The application navigates from the Home guest state to the customer-search page without authenticating the user.</t>
         </is>
       </c>
     </row>
@@ -627,14 +626,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Clean survey button
-Observe the destination page after navigation completes</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Clean survey button once
+Observe the destination view</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Selecting the Clean survey button transitions the application from the Home guest state to the vehicle-survey page without changing the unauthenticated session state.</t>
+          <t>The application navigates from the Home guest state to the vehicle-survey page while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -662,14 +661,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Click the Site survey button
-Observe the destination page after navigation completes</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Site survey button once
+Observe the destination view</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Selecting the Site survey button transitions the application from the Home guest state to the survey page while the user remains unauthenticated.</t>
+          <t>The application navigates from the Home guest state to the survey page while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -681,7 +680,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify returning to the Home page preserves guest-state behavior after opening the Login view</t>
+          <t>Verify navigation back to Home guest state after opening Login view from Person/Profile button</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -697,15 +696,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
 Click the Person/Profile button to open the Login page or Login view
-Use browser back navigation or the application Home navigation to return to the Home page
-Observe the Home page after returning</t>
+Use browser navigation or available SPA navigation to return to the Home page</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application returns to the shared Home page in guest state, approved guest controls remain visible and enabled, and the user is still unauthenticated.</t>
+          <t>The application returns to the Home page guest state and the approved guest-state controls remain visible and enabled without authenticating the user.</t>
         </is>
       </c>
     </row>
@@ -717,7 +715,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Home button remains visible and enabled in guest state</t>
+          <t>Verify navigation back to Home guest state after opening customer-search page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -733,14 +731,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Locate the Home button in the shared Home shell
-Select the Home button while already on the Home page</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Customer signup button
+Return to the Home page using approved application navigation</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Home button is visible and enabled in guest state and selecting it keeps the application on the Home page guest state without authentication changes.</t>
+          <t>The Home page guest state reloads successfully and the user remains unauthenticated with guest-state controls available.</t>
         </is>
       </c>
     </row>
@@ -752,7 +750,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Notification button remains visible and enabled in guest state</t>
+          <t>Verify navigation back to Home guest state after opening vehicle-survey page</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -768,14 +766,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Locate the Notification button in the shared Home shell
-Click the Notification button once</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Clean survey button
+Return to the Home page using approved application navigation</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Notification button is visible and enabled in guest state, and clicking it does not expose authenticated-only capabilities or change the unauthenticated session state.</t>
+          <t>The Home page guest state is restored and all approved guest-state controls remain visible and enabled.</t>
         </is>
       </c>
     </row>
@@ -787,7 +785,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Back button remains visible and enabled in guest state</t>
+          <t>Verify navigation back to Home guest state after opening survey page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -803,14 +801,156 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home while unauthenticated
-Locate the Back button in the shared Home shell
-Click the Back button from the Home page guest state</t>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Click the Site survey button
+Return to the Home page using approved application navigation</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Back button is visible and enabled in guest state and does not expose authenticated-only content or cause unauthorized navigation.</t>
+          <t>The Home page guest state reappears correctly and the session remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WT-HOME11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Verify Home button remains visible and enabled throughout guest-state navigation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Open the customer-search page using Customer signup button
+Return to the Home page guest state
+Observe the Home button availability</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>The Home button remains visible and enabled across guest-state navigation flows and continues to behave as a shared Home shell control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WT-HOME12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Verify Back button is visible and enabled in Home guest state</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Observe the Back button
+Click the Back button once</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>The Back button is visible and enabled in guest state and the application does not expose authenticated-only functionality after interaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WT-HOME13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Verify Notification button is visible and enabled in Home guest state</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Observe the Notification button
+Click the Notification button once</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>The Notification button is visible and enabled in guest state and no authenticated-only state becomes available after interaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WT-HOME14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Verify Home page remains in guest state after repeated navigation between guest-accessible pages</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
+Open the customer-search page and return to Home
+Open the vehicle-survey page and return to Home
+Open the survey page and return to Home</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Each navigation transition completes successfully and the Home page consistently returns in guest state without exposing authenticated-only controls or a logged-in user name button.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 35
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Home page loads successfully in guest state for an unauthenticated user</t>
+          <t>Verify Home page loads successfully in guest state from the approved entry URL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open a browser session
-Navigate to http://localhost/washtabui/home
-Wait for the Home page guest state to finish loading</t>
+          <t>Open the browser and navigate to http://localhost/washtabui/home
+Wait for the Home page to finish loading
+Observe the displayed Home page state before any login action</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state while the user remains unauthenticated and the shared Home page shell is visible.</t>
+          <t>The Home page loads successfully at http://localhost/washtabui/home in guest state with guest-accessible controls visible and no authenticated user state displayed.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify guest-state Home controls are visible and enabled on initial page load</t>
+          <t>Verify Person/Profile button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,14 +521,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button
-Attempt to focus and click each visible control once</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Locate the Person/Profile button on the Home page
+Observe the button state without clicking it</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are visible, enabled, focusable, and actionable in guest state.</t>
+          <t>The Person/Profile button is visible, enabled, clickable, and displayed as part of the Home page guest-state controls.</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify navigation from Person/Profile button opens the Login page or Login view from Home guest state</t>
+          <t>Verify Back button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,14 +556,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Person/Profile button once
-Observe the application transition</t>
+          <t>Launch the application in guest state
+Locate the Back button on the Home page
+Observe the Back button state</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Selecting the Person/Profile button transitions the application from Home guest state to the Login page or Login view while preserving unauthenticated state.</t>
+          <t>The Back button is visible and enabled while the application remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify navigation from Customer signup button opens the customer-search page</t>
+          <t>Verify Notification button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -591,14 +591,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Customer signup button once
-Observe the destination view</t>
+          <t>Launch the application in guest state
+Locate the Notification button on the Home page
+Observe the Notification button state</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application navigates from the Home guest state to the customer-search page without authenticating the user.</t>
+          <t>The Notification button is visible and enabled while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify navigation from Clean survey button opens the vehicle-survey page</t>
+          <t>Verify Home button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -626,14 +626,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Clean survey button once
-Observe the destination view</t>
+          <t>Launch the application in guest state
+Locate the Home button on the Home page
+Observe the Home button state</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates from the Home guest state to the vehicle-survey page while the user remains unauthenticated.</t>
+          <t>The Home button is visible and enabled while the application is in Home page guest state.</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify navigation from Site survey button opens the survey page</t>
+          <t>Verify Customer signup button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -661,14 +661,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Site survey button once
-Observe the destination view</t>
+          <t>Launch the application in guest state
+Locate the Customer signup button
+Observe the button state</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The application navigates from the Home guest state to the survey page while the user remains unauthenticated.</t>
+          <t>The Customer signup button is visible, enabled, and available for guest access.</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening Login view from Person/Profile button</t>
+          <t>Verify Clean survey button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -696,14 +696,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Person/Profile button to open the Login page or Login view
-Use browser navigation or available SPA navigation to return to the Home page</t>
+          <t>Launch the application in guest state
+Locate the Clean survey button
+Observe the button state</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and the approved guest-state controls remain visible and enabled without authenticating the user.</t>
+          <t>The Clean survey button is visible, enabled, and accessible to unauthenticated users.</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening customer-search page</t>
+          <t>Verify Site survey button is visible and enabled in guest state</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -731,14 +731,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Customer signup button
-Return to the Home page using approved application navigation</t>
+          <t>Launch the application in guest state
+Locate the Site survey button
+Observe the button state</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Home page guest state reloads successfully and the user remains unauthenticated with guest-state controls available.</t>
+          <t>The Site survey button is visible, enabled, and accessible in guest state.</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening vehicle-survey page</t>
+          <t>Verify navigation from Person/Profile button opens Login page or Login view</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -766,14 +766,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Clean survey button
-Return to the Home page using approved application navigation</t>
+          <t>Navigate to http://localhost/washtabui/home while unauthenticated
+Click the Person/Profile button once
+Observe the resulting application view</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Home page guest state is restored and all approved guest-state controls remain visible and enabled.</t>
+          <t>The application transitions from Home guest state to the Login page or Login view without authenticating the user.</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening survey page</t>
+          <t>Verify return to Home guest state after opening Login view from Person/Profile button</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -801,14 +801,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Click the Site survey button
-Return to the Home page using approved application navigation</t>
+          <t>Open the Login page or Login view using the Person/Profile button from Home guest state
+Navigate back to the Home page using browser navigation or application navigation
+Observe the Home page state after returning</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The Home page guest state reappears correctly and the session remains unauthenticated.</t>
+          <t>The application returns to the same Home page guest state with guest controls visible and without displaying authenticated user controls.</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify Home button remains visible and enabled throughout guest-state navigation</t>
+          <t>Verify Customer signup button navigates to customer-search page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -836,15 +836,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Open the customer-search page using Customer signup button
-Return to the Home page guest state
-Observe the Home button availability</t>
+          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
+Click the Customer signup button
+Observe the destination page or SPA view</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The Home button remains visible and enabled across guest-state navigation flows and continues to behave as a shared Home shell control.</t>
+          <t>The application navigates from the Home guest state to the customer-search page while the session remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -856,7 +855,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Back button is visible and enabled in Home guest state</t>
+          <t>Verify Clean survey button navigates to vehicle-survey page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -872,14 +871,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Back button
-Click the Back button once</t>
+          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
+Click the Clean survey button
+Observe the destination page or SPA view</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The Back button is visible and enabled in guest state and the application does not expose authenticated-only functionality after interaction.</t>
+          <t>The application navigates from the Home guest state to the vehicle-survey page without requiring login.</t>
         </is>
       </c>
     </row>
@@ -891,7 +890,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Notification button is visible and enabled in Home guest state</t>
+          <t>Verify Site survey button navigates to survey page</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -907,14 +906,14 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Observe the Notification button
-Click the Notification button once</t>
+          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
+Click the Site survey button
+Observe the destination page or SPA view</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The Notification button is visible and enabled in guest state and no authenticated-only state becomes available after interaction.</t>
+          <t>The application navigates from the Home guest state to the survey page while remaining in unauthenticated mode.</t>
         </is>
       </c>
     </row>
@@ -926,12 +925,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify Home page remains in guest state after repeated navigation between guest-accessible pages</t>
+          <t>Verify Home button interaction preserves guest-state session</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -942,15 +941,189 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as an unauthenticated user
-Open the customer-search page and return to Home
-Open the vehicle-survey page and return to Home
-Open the survey page and return to Home</t>
+          <t>Launch the application in guest state
+Click the Home button
+Observe the resulting page state</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Each navigation transition completes successfully and the Home page consistently returns in guest state without exposing authenticated-only controls or a logged-in user name button.</t>
+          <t>The application remains on or returns to the Home page guest state without authenticating the user or hiding guest controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WT-HOME15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Verify Notification button interaction does not expose authenticated functionality to guest users</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Launch the application in guest state
+Click the Notification button
+Observe any resulting behavior or displayed content</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>The Notification button does not expose authenticated-only functionality and the application remains in guest-accessible state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT-HOME16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verify Back button interaction does not incorrectly authenticate the guest user</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Launch the application in guest state
+Click the Back button
+Observe the resulting application state</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>The application does not enter an authenticated state and no logged-in user controls become visible after using the Back button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WT-HOME17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Verify guest-accessible controls remain available after returning from customer-search page</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Navigate to the customer-search page using the Customer signup button
+Return to the Home page guest state
+Inspect the guest-state controls on the Home page</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>The Home page displays the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button as visible and enabled after returning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WT-HOME18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Verify guest-accessible controls remain available after returning from vehicle-survey page</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Navigate to the vehicle-survey page using the Clean survey button
+Return to the Home page guest state
+Inspect all guest-state controls</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>The Home page returns to guest state with all approved guest-accessible controls visible and enabled and without authenticated user indicators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WT-HOME19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Verify guest-accessible controls remain available after returning from survey page</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Navigate to the survey page using the Site survey button
+Return to the Home page guest state
+Inspect the Home page controls</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>The Home page guest state is restored with approved guest controls accessible and authenticated-only controls still absent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 39
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Home page loads successfully in guest state from the approved application URL</t>
+          <t>Verify guest user can directly access the Home page using the approved entry URL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open a browser session
-Navigate to http://localhost/washtabui/home
-Wait for the Home page guest state to finish loading</t>
+          <t>Launch the application in a new browser session.
+Navigate directly to http://localhost/washtabui/home.
+Wait for the Home page to finish loading.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Home page loads successfully in guest state at the approved URL while the user remains unauthenticated and the shared Home page shell is visible.</t>
+          <t>The application loads successfully at http://localhost/washtabui/home and displays the Home page in guest state without requiring authentication or redirecting to another page.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify guest-state controls and shared Home shell controls are visible and enabled on initial Home page load</t>
+          <t>Verify Person/Profile button is visible and enabled on the Home page in guest state</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,15 +521,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Observe the Home page guest state after load completion
-Verify the Person/Profile button, Back button, Notification button, Home button, Customer signup button, Clean survey button, and Site survey button are visible
-Verify each approved button is enabled and clickable</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Observe the Person/Profile button on the Home page.
+Check that the button is visible and enabled before interaction.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved guest-state controls and shared Home shell controls are visible, enabled, and actionable in the Home page guest state.</t>
+          <t>The Person/Profile button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -541,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button navigates from Home guest state to the Login page or Login view</t>
+          <t>Verify Back button is visible and enabled on the Home page in guest state</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -557,14 +556,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Verify the Home page guest state is displayed
-Click the Person/Profile button once</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Observe the Back button on the Home page.
+Check that the button is visible and enabled before interaction.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page guest state to the Login page or Login view while navigation clearly originates from the Home page.</t>
+          <t>The Back button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -576,7 +575,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Customer signup button navigates from Home guest state to the customer-search page</t>
+          <t>Verify Notification button is visible and enabled on the Home page in guest state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -592,14 +591,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Verify the Home page guest state is displayed
-Click the Customer signup button once</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Observe the Notification button on the Home page.
+Check that the button is visible and enabled before interaction.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The customer-search page opens from the Home page guest state and the user remains unauthenticated throughout the transition.</t>
+          <t>The Notification button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -611,7 +610,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Clean survey button navigates from Home guest state to the vehicle-survey page</t>
+          <t>Verify Home button is visible and enabled on the Home page in guest state</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -627,14 +626,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Verify the Home page guest state is displayed
-Click the Clean survey button once</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Observe the Home button on the Home page.
+Check that the button is visible and enabled before interaction.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The vehicle-survey page opens from the Home page guest state and the user remains unauthenticated throughout the transition.</t>
+          <t>The Home button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -646,7 +645,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify Site survey button navigates from Home guest state to the survey page</t>
+          <t>Verify Customer signup button is visible and enabled on the Home page in guest state</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -662,14 +661,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Verify the Home page guest state is displayed
-Click the Site survey button once</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Observe the Customer signup button on the Home page.
+Check that the button is visible and enabled before interaction.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The survey page opens from the Home page guest state and the user remains unauthenticated throughout the transition.</t>
+          <t>The Customer signup button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -681,7 +680,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify Home button remains visible and enabled in guest state</t>
+          <t>Verify Clean survey button is visible and enabled on the Home page in guest state</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -697,14 +696,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Locate the Home button on the shared Home shell
-Verify the Home button is visible and enabled</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Observe the Clean survey button on the Home page.
+Check that the button is visible and enabled before interaction.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The Home button is displayed in the Home page guest state and is enabled for interaction.</t>
+          <t>The Clean survey button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -716,7 +715,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Back button remains visible and enabled in guest state</t>
+          <t>Verify Site survey button is visible and enabled on the Home page in guest state</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -732,14 +731,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Locate the Back button on the shared Home shell
-Verify the Back button is visible and enabled</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Observe the Site survey button on the Home page.
+Check that the button is visible and enabled before interaction.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Back button is displayed in the Home page guest state and is enabled for interaction.</t>
+          <t>The Site survey button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
         </is>
       </c>
     </row>
@@ -751,7 +750,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify Notification button remains visible and enabled in guest state</t>
+          <t>Verify clicking the Person/Profile button navigates guest user to the login URL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -767,14 +766,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Locate the Notification button on the shared Home shell
-Verify the Notification button is visible and enabled</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Click the Person/Profile button once.
+Observe the browser URL after navigation completes.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The Notification button is displayed in the Home page guest state and is enabled for interaction.</t>
+          <t>The application navigates from the Home page to the login page and the browser URL equals /washtabui/login?data=undefined.</t>
         </is>
       </c>
     </row>
@@ -786,7 +785,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening the Login view from the Person/Profile button</t>
+          <t>Verify clicking the Customer signup button navigates guest user to customer-search page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -802,14 +801,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Click the Person/Profile button to open the Login page or Login view
-Use browser back navigation or approved application return navigation to return to Home</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Click the Customer signup button once.
+Observe the browser URL after navigation completes.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state and approved guest-state controls are visible again without authenticating the user.</t>
+          <t>The application navigates from the Home page to the customer-search page and the browser URL contains /customer-search.</t>
         </is>
       </c>
     </row>
@@ -821,7 +820,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening the customer-search page</t>
+          <t>Verify clicking the Clean survey button navigates guest user to vehicle-survey page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -837,14 +836,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Click the Customer signup button
-Return to the Home page using browser back navigation or approved application navigation</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Click the Clean survey button once.
+Observe the browser URL after navigation completes.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state with approved guest-state controls visible and the user still unauthenticated.</t>
+          <t>The application navigates from the Home page to the vehicle-survey page and the browser URL contains vehicle-survey.</t>
         </is>
       </c>
     </row>
@@ -856,7 +855,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening the vehicle-survey page</t>
+          <t>Verify clicking the Site survey button navigates guest user to survey page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -872,14 +871,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Click the Clean survey button
-Return to the Home page using browser back navigation or approved application navigation</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Click the Site survey button once.
+Observe the browser URL after navigation completes.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state with approved guest-state controls visible and the user still unauthenticated.</t>
+          <t>The application navigates from the Home page to the survey page and the browser URL contains survey?data.</t>
         </is>
       </c>
     </row>
@@ -891,7 +890,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify navigation back to Home guest state after opening the survey page</t>
+          <t>Verify all approved Home page navigation controls are enabled and interactive before user interaction</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -907,14 +906,120 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Launch the application at http://localhost/washtabui/home while unauthenticated
-Click the Site survey button
-Return to the Home page using browser back navigation or approved application navigation</t>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Inspect the Person/Profile, Back, Notification, Home, Customer signup, Clean survey, and Site survey buttons.
+Attempt focus and click readiness checks without leaving the page.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The application returns to the Home page guest state with approved guest-state controls visible and the user still unauthenticated.</t>
+          <t>All approved Home page navigation buttons are enabled, focusable, and interactive before any workflow navigation occurs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WT-HOME14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Verify Home button remains interactive and does not redirect away from the Home page unexpectedly</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Click the Home button once.
+Observe the browser URL and rendered page state.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>The Home button remains interactive and the user stays on or returns to the Home page at http://localhost/washtabui/home without entering an invalid navigation state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WT-HOME15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Verify Back button interaction from initial Home page state does not break the guest Home workflow</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Open a fresh browser session.
+Navigate directly to http://localhost/washtabui/home.
+Click the Back button on the Home page.
+Observe the resulting browser state.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>The application handles the Back button interaction gracefully without displaying an application error or broken page state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT-HOME16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verify Notification button interaction is accepted while user remains in guest-accessible workflow state</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+Click the Notification button once.
+Observe the application response and page stability.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>The Notification button is interactive and the application remains stable without rendering a broken page or unexpected authentication failure.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 40
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify guest user can directly access the Home page using the approved entry URL</t>
+          <t>Verify guest user can directly access the Home page URL and Home page loads successfully</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,15 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application in a new browser session.
+          <t>Launch the application in a browser session.
 Navigate directly to http://localhost/washtabui/home.
-Wait for the Home page to finish loading.</t>
+Wait for the Home page to complete loading.
+Observe the displayed page state without authenticating.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application loads successfully at http://localhost/washtabui/home and displays the Home page in guest state without requiring authentication or redirecting to another page.</t>
+          <t>The application loads successfully at http://localhost/washtabui/home and displays the Home page in guest state without redirecting to authentication or showing access denial.</t>
         </is>
       </c>
     </row>
@@ -521,14 +522,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Observe the Person/Profile button on the Home page.
-Check that the button is visible and enabled before interaction.</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page to load completely.
+Locate the Person/Profile button.
+Observe the visibility and enabled state of the Person/Profile button.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Person/Profile button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
+          <t>The Person/Profile button is visible, enabled, and available for interaction on the Home page in guest state.</t>
         </is>
       </c>
     </row>
@@ -556,14 +558,15 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Observe the Back button on the Home page.
-Check that the button is visible and enabled before interaction.</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page to load completely.
+Locate the Back button.
+Observe the visibility and enabled state of the Back button.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Back button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
+          <t>The Back button is visible, enabled, and available for interaction on the Home page in guest state.</t>
         </is>
       </c>
     </row>
@@ -591,14 +594,15 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Observe the Notification button on the Home page.
-Check that the button is visible and enabled before interaction.</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page to load completely.
+Locate the Notification button.
+Observe the visibility and enabled state of the Notification button.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The Notification button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
+          <t>The Notification button is visible, enabled, and available for interaction on the Home page in guest state.</t>
         </is>
       </c>
     </row>
@@ -626,14 +630,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Observe the Home button on the Home page.
-Check that the button is visible and enabled before interaction.</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page to load completely.
+Locate the Home button.
+Observe the visibility and enabled state of the Home button.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The Home button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
+          <t>The Home button is visible, enabled, and available for interaction on the Home page in guest state.</t>
         </is>
       </c>
     </row>
@@ -661,14 +666,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Observe the Customer signup button on the Home page.
-Check that the button is visible and enabled before interaction.</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page to load completely.
+Locate the Customer signup button.
+Observe the visibility and enabled state of the Customer signup button.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The Customer signup button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
+          <t>The Customer signup button is visible, enabled, and available for interaction on the Home page in guest state.</t>
         </is>
       </c>
     </row>
@@ -696,14 +702,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Observe the Clean survey button on the Home page.
-Check that the button is visible and enabled before interaction.</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page to load completely.
+Locate the Clean survey button.
+Observe the visibility and enabled state of the Clean survey button.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The Clean survey button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
+          <t>The Clean survey button is visible, enabled, and available for interaction on the Home page in guest state.</t>
         </is>
       </c>
     </row>
@@ -731,14 +738,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Observe the Site survey button on the Home page.
-Check that the button is visible and enabled before interaction.</t>
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page to load completely.
+Locate the Site survey button.
+Observe the visibility and enabled state of the Site survey button.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Site survey button is visible, enabled, and interactive on the Home page while the user remains in guest state.</t>
+          <t>The Site survey button is visible, enabled, and available for interaction on the Home page in guest state.</t>
         </is>
       </c>
     </row>
@@ -750,7 +758,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify clicking the Person/Profile button navigates guest user to the login URL</t>
+          <t>Verify clicking the Person/Profile button navigates the guest user to the login page URL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -766,14 +774,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page controls to become interactive.
 Click the Person/Profile button once.
-Observe the browser URL after navigation completes.</t>
+Observe the resulting browser URL.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The application navigates from the Home page to the login page and the browser URL equals /washtabui/login?data=undefined.</t>
+          <t>The application transitions from the Home page to the login page and the resulting URL is exactly /washtabui/login?data=undefined.</t>
         </is>
       </c>
     </row>
@@ -785,7 +794,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify clicking the Customer signup button navigates guest user to customer-search page</t>
+          <t>Verify clicking the Customer signup button navigates the guest user to the customer-search workflow entry page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -801,14 +810,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page controls to become interactive.
 Click the Customer signup button once.
-Observe the browser URL after navigation completes.</t>
+Observe the resulting browser URL.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application navigates from the Home page to the customer-search page and the browser URL contains /customer-search.</t>
+          <t>The application transitions from the Home page to the customer-search workflow entry page and the resulting URL contains /customer-search.</t>
         </is>
       </c>
     </row>
@@ -820,7 +830,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify clicking the Clean survey button navigates guest user to vehicle-survey page</t>
+          <t>Verify clicking the Clean survey button navigates the guest user to the vehicle-survey workflow entry page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -836,14 +846,15 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page controls to become interactive.
 Click the Clean survey button once.
-Observe the browser URL after navigation completes.</t>
+Observe the resulting browser URL.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application navigates from the Home page to the vehicle-survey page and the browser URL contains vehicle-survey.</t>
+          <t>The application transitions from the Home page to the vehicle-survey workflow entry page and the resulting URL contains vehicle-survey.</t>
         </is>
       </c>
     </row>
@@ -855,7 +866,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify clicking the Site survey button navigates guest user to survey page</t>
+          <t>Verify clicking the Site survey button navigates the guest user to the survey workflow entry page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -871,155 +882,15 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
+          <t>Navigate to http://localhost/washtabui/home as a guest user.
+Wait for the Home page controls to become interactive.
 Click the Site survey button once.
-Observe the browser URL after navigation completes.</t>
+Observe the resulting browser URL.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application navigates from the Home page to the survey page and the browser URL contains survey?data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>WT-HOME13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Verify all approved Home page navigation controls are enabled and interactive before user interaction</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Inspect the Person/Profile, Back, Notification, Home, Customer signup, Clean survey, and Site survey buttons.
-Attempt focus and click readiness checks without leaving the page.</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>All approved Home page navigation buttons are enabled, focusable, and interactive before any workflow navigation occurs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>WT-HOME14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Verify Home button remains interactive and does not redirect away from the Home page unexpectedly</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Click the Home button once.
-Observe the browser URL and rendered page state.</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>The Home button remains interactive and the user stays on or returns to the Home page at http://localhost/washtabui/home without entering an invalid navigation state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>WT-HOME15</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Verify Back button interaction from initial Home page state does not break the guest Home workflow</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Open a fresh browser session.
-Navigate directly to http://localhost/washtabui/home.
-Click the Back button on the Home page.
-Observe the resulting browser state.</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>The application handles the Back button interaction gracefully without displaying an application error or broken page state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>WT-HOME16</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Verify Notification button interaction is accepted while user remains in guest-accessible workflow state</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Navigate directly to http://localhost/washtabui/home in guest state.
-Click the Notification button once.
-Observe the application response and page stability.</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>The Notification button is interactive and the application remains stable without rendering a broken page or unexpected authentication failure.</t>
+          <t>The application transitions from the Home page to the survey workflow entry page and the resulting URL contains survey?data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 41
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify guest user can directly access the Home page URL and Home page loads successfully</t>
+          <t>Verify guest user can directly access the Home page using the approved entry URL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,15 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application in a browser session.
+          <t>Launch the application in a new browser session.
 Navigate directly to http://localhost/washtabui/home.
-Wait for the Home page to complete loading.
-Observe the displayed page state without authenticating.</t>
+Wait for the Home page to finish loading.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application loads successfully at http://localhost/washtabui/home and displays the Home page in guest state without redirecting to authentication or showing access denial.</t>
+          <t>The application loads the Home page successfully in guest state without requiring authentication and the browser URL remains http://localhost/washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -522,15 +521,13 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page to load completely.
-Locate the Person/Profile button.
-Observe the visibility and enabled state of the Person/Profile button.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Observe the Person/Profile button on the Home page.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Person/Profile button is visible, enabled, and available for interaction on the Home page in guest state.</t>
+          <t>The Person/Profile button is visible, enabled, and interactive before user interaction begins.</t>
         </is>
       </c>
     </row>
@@ -558,15 +555,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page to load completely.
-Locate the Back button.
-Observe the visibility and enabled state of the Back button.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Observe the Back button on the Home page.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Back button is visible, enabled, and available for interaction on the Home page in guest state.</t>
+          <t>The Back button is visible, enabled, and interactive before user interaction begins.</t>
         </is>
       </c>
     </row>
@@ -594,15 +589,13 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page to load completely.
-Locate the Notification button.
-Observe the visibility and enabled state of the Notification button.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Observe the Notification button on the Home page.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The Notification button is visible, enabled, and available for interaction on the Home page in guest state.</t>
+          <t>The Notification button is visible, enabled, and interactive before user interaction begins.</t>
         </is>
       </c>
     </row>
@@ -630,15 +623,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page to load completely.
-Locate the Home button.
-Observe the visibility and enabled state of the Home button.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Observe the Home button on the Home page.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The Home button is visible, enabled, and available for interaction on the Home page in guest state.</t>
+          <t>The Home button is visible, enabled, and interactive before user interaction begins.</t>
         </is>
       </c>
     </row>
@@ -666,15 +657,13 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page to load completely.
-Locate the Customer signup button.
-Observe the visibility and enabled state of the Customer signup button.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Observe the Customer signup button on the Home page.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The Customer signup button is visible, enabled, and available for interaction on the Home page in guest state.</t>
+          <t>The Customer signup button is visible, enabled, and interactive before user interaction begins.</t>
         </is>
       </c>
     </row>
@@ -702,15 +691,13 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page to load completely.
-Locate the Clean survey button.
-Observe the visibility and enabled state of the Clean survey button.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Observe the Clean survey button on the Home page.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The Clean survey button is visible, enabled, and available for interaction on the Home page in guest state.</t>
+          <t>The Clean survey button is visible, enabled, and interactive before user interaction begins.</t>
         </is>
       </c>
     </row>
@@ -738,15 +725,13 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page to load completely.
-Locate the Site survey button.
-Observe the visibility and enabled state of the Site survey button.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Observe the Site survey button on the Home page.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>The Site survey button is visible, enabled, and available for interaction on the Home page in guest state.</t>
+          <t>The Site survey button is visible, enabled, and interactive before user interaction begins.</t>
         </is>
       </c>
     </row>
@@ -758,7 +743,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify clicking the Person/Profile button navigates the guest user to the login page URL</t>
+          <t>Verify selecting the Person/Profile button navigates the guest user to the login page URL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -774,15 +759,13 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page controls to become interactive.
-Click the Person/Profile button once.
-Observe the resulting browser URL.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Click the Person/Profile button once.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page to the login page and the resulting URL is exactly /washtabui/login?data=undefined.</t>
+          <t>The application transitions from the Home page to the login page and the browser URL equals /washtabui/login?data=undefined.</t>
         </is>
       </c>
     </row>
@@ -794,7 +777,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify clicking the Customer signup button navigates the guest user to the customer-search workflow entry page</t>
+          <t>Verify selecting the Customer signup button navigates the guest user to the customer-search workflow entry URL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -810,15 +793,13 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page controls to become interactive.
-Click the Customer signup button once.
-Observe the resulting browser URL.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Click the Customer signup button once.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page to the customer-search workflow entry page and the resulting URL contains /customer-search.</t>
+          <t>The application transitions from the Home page to the customer-search workflow and the resulting URL contains /customer-search.</t>
         </is>
       </c>
     </row>
@@ -830,7 +811,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify clicking the Clean survey button navigates the guest user to the vehicle-survey workflow entry page</t>
+          <t>Verify selecting the Clean survey button navigates the guest user to the vehicle-survey workflow entry URL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -846,15 +827,13 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page controls to become interactive.
-Click the Clean survey button once.
-Observe the resulting browser URL.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Click the Clean survey button once.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page to the vehicle-survey workflow entry page and the resulting URL contains vehicle-survey.</t>
+          <t>The application transitions from the Home page to the vehicle-survey workflow and the resulting URL contains vehicle-survey.</t>
         </is>
       </c>
     </row>
@@ -866,7 +845,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify clicking the Site survey button navigates the guest user to the survey workflow entry page</t>
+          <t>Verify selecting the Site survey button navigates the guest user to the survey workflow entry URL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -882,15 +861,13 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home as a guest user.
-Wait for the Home page controls to become interactive.
-Click the Site survey button once.
-Observe the resulting browser URL.</t>
+          <t>Navigate directly to http://localhost/washtabui/home.
+Click the Site survey button once.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page to the survey workflow entry page and the resulting URL contains survey?data.</t>
+          <t>The application transitions from the Home page to the survey workflow and the resulting URL contains survey?data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 43
</commit_message>
<xml_diff>
--- a/manual_tests/home/home_approved_manual_tests.xlsx
+++ b/manual_tests/home/home_approved_manual_tests.xlsx
@@ -488,7 +488,7 @@
         <is>
           <t>Launch the application in a new browser session.
 Navigate directly to http://localhost/washtabui/home.
-Wait for the Home page to fully load.</t>
+Wait for the Home page to complete loading.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Person/Profile button navigates guest user to login page URL</t>
+          <t>Verify clicking the Person/Profile button navigates guest user to the login page URL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,14 +521,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state.
+          <t>Navigate directly to http://localhost/washtabui/home.
 Click the Person/Profile button once.
-Observe the browser URL after navigation completes.</t>
+Observe the resulting URL in the browser.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The application navigates from the Home page to the login page and the URL equals /washtabui/login?data=undefined.</t>
+          <t>The application transitions from the Home page to the Login page and the browser URL equals /washtabui/login?data=undefined.</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Customer signup button navigates guest user to customer-search page</t>
+          <t>Verify clicking the Customer signup button navigates guest user to customer-search workflow entry</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,14 +556,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state.
+          <t>Navigate directly to http://localhost/washtabui/home.
 Click the Customer signup button once.
-Observe the browser URL after navigation completes.</t>
+Observe the resulting URL in the browser.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The application navigates from the Home page to the customer-search workflow and the resulting URL contains /customer-search.</t>
+          <t>The application transitions from the Home page to the customer-search workflow entry page and the browser URL contains /customer-search.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify Clean survey button navigates guest user to vehicle-survey page</t>
+          <t>Verify clicking the Clean survey button navigates guest user to vehicle-survey workflow entry</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -591,14 +591,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state.
+          <t>Navigate directly to http://localhost/washtabui/home.
 Click the Clean survey button once.
-Observe the browser URL after navigation completes.</t>
+Observe the resulting URL in the browser.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application navigates from the Home page to the vehicle survey workflow and the resulting URL contains vehicle-survey.</t>
+          <t>The application transitions from the Home page to the vehicle-survey workflow entry page and the browser URL contains vehicle-survey.</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify Site survey button navigates guest user to survey page</t>
+          <t>Verify clicking the Site survey button navigates guest user to survey workflow entry</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -626,14 +626,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state.
+          <t>Navigate directly to http://localhost/washtabui/home.
 Click the Site survey button once.
-Observe the browser URL after navigation completes.</t>
+Observe the resulting URL in the browser.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The application navigates from the Home page to the survey workflow and the resulting URL contains survey?data.</t>
+          <t>The application transitions from the Home page to the survey workflow entry page and the browser URL contains survey?data.</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify all approved Home page navigation controls are enabled before interaction</t>
+          <t>Verify all approved Home page navigation controls are enabled together after page load</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -662,13 +662,12 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>Navigate directly to http://localhost/washtabui/home.
-Wait for the Home page to finish loading.
-Attempt to focus or hover over each approved navigation control.</t>
+Attempt to focus or interact with each approved Home page button without leaving the page.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>All approved Home page navigation buttons are enabled, interactive, and available for user action before navigation begins.</t>
+          <t>All approved Home page buttons accept interaction and none of the controls appear disabled, blocked, or non-clickable.</t>
         </is>
       </c>
     </row>

</xml_diff>